<commit_message>
fix(mobile): remove onboarding language step; explain refused phone numbers
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0185gN8jDyiGGwA6x5BUeZUi
</commit_message>
<xml_diff>
--- a/apps/api/prisma/seed/translations_seed.xlsx
+++ b/apps/api/prisma/seed/translations_seed.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="822" uniqueCount="763">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="828" uniqueCount="769">
   <si>
     <t>key</t>
   </si>
@@ -2300,6 +2300,24 @@
   </si>
   <si>
     <t>Клиенты видят ваше полное имя в профиле — укажите его как в лицензии.</t>
+  </si>
+  <si>
+    <t>error.api.PHONE_INVALID_US</t>
+  </si>
+  <si>
+    <t>This isn't a valid US number. Check the area code, e.g. (202) 555-1234.</t>
+  </si>
+  <si>
+    <t>Такого номера США нет. Проверьте код города, например (202) 555-1234.</t>
+  </si>
+  <si>
+    <t>error.api.PHONE_TYPE_NOT_ALLOWED</t>
+  </si>
+  <si>
+    <t>We can't text this number. Please use a US mobile number.</t>
+  </si>
+  <si>
+    <t>На этот номер нельзя отправить SMS. Укажите мобильный номер США.</t>
   </si>
 </sst>
 </file>
@@ -2676,7 +2694,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C274"/>
+  <dimension ref="A1:C276"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -5697,6 +5715,28 @@
         <v>762</v>
       </c>
     </row>
+    <row r="275" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A275" t="s">
+        <v>763</v>
+      </c>
+      <c r="B275" t="s">
+        <v>764</v>
+      </c>
+      <c r="C275" t="s">
+        <v>765</v>
+      </c>
+    </row>
+    <row r="276" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A276" t="s">
+        <v>766</v>
+      </c>
+      <c r="B276" t="s">
+        <v>767</v>
+      </c>
+      <c r="C276" t="s">
+        <v>768</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>

</xml_diff>

<commit_message>
feat(mobile): consents step as role-style cards, compact document grid, no optional consents (owner request)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0185gN8jDyiGGwA6x5BUeZUi
</commit_message>
<xml_diff>
--- a/apps/api/prisma/seed/translations_seed.xlsx
+++ b/apps/api/prisma/seed/translations_seed.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1032" uniqueCount="942">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1062" uniqueCount="972">
   <si>
     <t>key</t>
   </si>
@@ -2837,6 +2837,96 @@
   </si>
   <si>
     <t>account.flow.done.action</t>
+  </si>
+  <si>
+    <t>error.api.DEVICE_ATTESTATION_REQUIRED</t>
+  </si>
+  <si>
+    <t>We couldn't verify this device. Update the app from the App Store or Google Play and try again.</t>
+  </si>
+  <si>
+    <t>Не удалось проверить устройство. Обновите приложение из App Store или Google Play и попробуйте снова.</t>
+  </si>
+  <si>
+    <t>error.api.AUTH_REFRESH_REUSE_DETECTED</t>
+  </si>
+  <si>
+    <t>For your security, you've been signed out on all devices. Please sign in again.</t>
+  </si>
+  <si>
+    <t>В целях безопасности выполнен выход на всех устройствах. Войдите снова.</t>
+  </si>
+  <si>
+    <t>error.api.AUTH_SESSION_REVOKED</t>
+  </si>
+  <si>
+    <t>Your session has ended. Please sign in again.</t>
+  </si>
+  <si>
+    <t>Сеанс завершён. Войдите снова.</t>
+  </si>
+  <si>
+    <t>error.api.IDEMPOTENCY_KEY_CONFLICT</t>
+  </si>
+  <si>
+    <t>This request is already being processed. Please wait a moment.</t>
+  </si>
+  <si>
+    <t>Запрос уже обрабатывается. Подождите немного.</t>
+  </si>
+  <si>
+    <t>error.api.FORBIDDEN</t>
+  </si>
+  <si>
+    <t>You don't have access to this action.</t>
+  </si>
+  <si>
+    <t>У вас нет доступа к этому действию.</t>
+  </si>
+  <si>
+    <t>error.api.NOT_FOUND</t>
+  </si>
+  <si>
+    <t>Not found. It may have been removed.</t>
+  </si>
+  <si>
+    <t>Не найдено. Возможно, это было удалено.</t>
+  </si>
+  <si>
+    <t>error.api.NOT_IMPLEMENTED</t>
+  </si>
+  <si>
+    <t>This feature isn't available yet.</t>
+  </si>
+  <si>
+    <t>Эта функция пока недоступна.</t>
+  </si>
+  <si>
+    <t>onboarding.consents.age18.desc</t>
+  </si>
+  <si>
+    <t>LawBid is available to adults only.</t>
+  </si>
+  <si>
+    <t>LawBid доступен только совершеннолетним.</t>
+  </si>
+  <si>
+    <t>onboarding.consents.terms.desc</t>
+  </si>
+  <si>
+    <t>You can read the documents below.</t>
+  </si>
+  <si>
+    <t>Документы можно прочитать ниже.</t>
+  </si>
+  <si>
+    <t>onboarding.consents.docs</t>
+  </si>
+  <si>
+    <t>Documents</t>
+  </si>
+  <si>
+    <t>Документы</t>
   </si>
 </sst>
 </file>
@@ -3213,7 +3303,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C344"/>
+  <dimension ref="A1:C354"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -7004,6 +7094,116 @@
         <v>357</v>
       </c>
     </row>
+    <row r="345" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A345" t="s">
+        <v>942</v>
+      </c>
+      <c r="B345" t="s">
+        <v>943</v>
+      </c>
+      <c r="C345" t="s">
+        <v>944</v>
+      </c>
+    </row>
+    <row r="346" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A346" t="s">
+        <v>945</v>
+      </c>
+      <c r="B346" t="s">
+        <v>946</v>
+      </c>
+      <c r="C346" t="s">
+        <v>947</v>
+      </c>
+    </row>
+    <row r="347" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A347" t="s">
+        <v>948</v>
+      </c>
+      <c r="B347" t="s">
+        <v>949</v>
+      </c>
+      <c r="C347" t="s">
+        <v>950</v>
+      </c>
+    </row>
+    <row r="348" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A348" t="s">
+        <v>951</v>
+      </c>
+      <c r="B348" t="s">
+        <v>952</v>
+      </c>
+      <c r="C348" t="s">
+        <v>953</v>
+      </c>
+    </row>
+    <row r="349" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A349" t="s">
+        <v>954</v>
+      </c>
+      <c r="B349" t="s">
+        <v>955</v>
+      </c>
+      <c r="C349" t="s">
+        <v>956</v>
+      </c>
+    </row>
+    <row r="350" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A350" t="s">
+        <v>957</v>
+      </c>
+      <c r="B350" t="s">
+        <v>958</v>
+      </c>
+      <c r="C350" t="s">
+        <v>959</v>
+      </c>
+    </row>
+    <row r="351" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A351" t="s">
+        <v>960</v>
+      </c>
+      <c r="B351" t="s">
+        <v>961</v>
+      </c>
+      <c r="C351" t="s">
+        <v>962</v>
+      </c>
+    </row>
+    <row r="352" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A352" t="s">
+        <v>963</v>
+      </c>
+      <c r="B352" t="s">
+        <v>964</v>
+      </c>
+      <c r="C352" t="s">
+        <v>965</v>
+      </c>
+    </row>
+    <row r="353" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A353" t="s">
+        <v>966</v>
+      </c>
+      <c r="B353" t="s">
+        <v>967</v>
+      </c>
+      <c r="C353" t="s">
+        <v>968</v>
+      </c>
+    </row>
+    <row r="354" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A354" t="s">
+        <v>969</v>
+      </c>
+      <c r="B354" t="s">
+        <v>970</v>
+      </c>
+      <c r="C354" t="s">
+        <v>971</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>

</xml_diff>

<commit_message>
fix(mobile): bind email magic link to the requesting device
Security review 2026-09-27 (High): magic links no longer carry email +
OTP code. Email login-code requests now send linkChallenge =
base64url(SHA-256(verifier)); the 32-byte verifier stays in
flutter_secure_storage and is cleared on sign-in/logout. Links are
lawbid://auth/email-code?token=<43 base64url> (or https lawbid.app) and
are redeemed via POST /auth/otp/verify-link with token + verifier. With
no stored verifier the app makes no request and shows the email step
with auth.magicLink.otherDevice. Includes the regenerated lawbid_api
client (verifyOtpLink, OtpVerifyLinkDto, linkChallenge).

Also: consents documents grid - an odd last item spans the full width
(owner request); consents goldens regenerated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0185gN8jDyiGGwA6x5BUeZUi
</commit_message>
<xml_diff>
--- a/apps/api/prisma/seed/translations_seed.xlsx
+++ b/apps/api/prisma/seed/translations_seed.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1062" uniqueCount="972">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1065" uniqueCount="975">
   <si>
     <t>key</t>
   </si>
@@ -2927,6 +2927,15 @@
   </si>
   <si>
     <t>Документы</t>
+  </si>
+  <si>
+    <t>auth.magicLink.otherDevice</t>
+  </si>
+  <si>
+    <t>Open the link on the phone where you requested the code, or enter the code from the email.</t>
+  </si>
+  <si>
+    <t>Откройте ссылку на телефоне, где вы запрашивали код, или введите код из письма.</t>
   </si>
 </sst>
 </file>
@@ -3303,7 +3312,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C354"/>
+  <dimension ref="A1:C355"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -7204,6 +7213,17 @@
         <v>971</v>
       </c>
     </row>
+    <row r="355" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A355" t="s">
+        <v>972</v>
+      </c>
+      <c r="B355" t="s">
+        <v>973</v>
+      </c>
+      <c r="C355" t="s">
+        <v>974</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>

</xml_diff>

<commit_message>
chore: merge 3.3/3.4 translations and regenerated contract
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0185gN8jDyiGGwA6x5BUeZUi
</commit_message>
<xml_diff>
--- a/apps/api/prisma/seed/translations_seed.xlsx
+++ b/apps/api/prisma/seed/translations_seed.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1116" uniqueCount="1026">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1185" uniqueCount="1095">
   <si>
     <t>key</t>
   </si>
@@ -3089,6 +3089,213 @@
   </si>
   <si>
     <t>Загрузка файлов сейчас недоступна. Попробуйте позже.</t>
+  </si>
+  <si>
+    <t>error.api.VERIFICATION_ALREADY_PENDING</t>
+  </si>
+  <si>
+    <t>You already have a verification request. Continue it or wait for the decision.</t>
+  </si>
+  <si>
+    <t>У вас уже есть заявка на верификацию. Продолжите её или дождитесь решения.</t>
+  </si>
+  <si>
+    <t>error.api.VERIFICATION_SUBMISSION_LIMIT</t>
+  </si>
+  <si>
+    <t>Too many requests in the last 30 days. Please try again later.</t>
+  </si>
+  <si>
+    <t>Слишком много заявок за 30 дней. Попробуйте позже.</t>
+  </si>
+  <si>
+    <t>error.api.VERIFICATION_INVALID_STATUS</t>
+  </si>
+  <si>
+    <t>This request can't be changed right now. Please refresh.</t>
+  </si>
+  <si>
+    <t>Сейчас заявку нельзя изменить. Обновите экран.</t>
+  </si>
+  <si>
+    <t>error.api.VERIFICATION_INCOMPLETE</t>
+  </si>
+  <si>
+    <t>Your request is incomplete: add a license with its document, an ID document and a selfie.</t>
+  </si>
+  <si>
+    <t>Заявка не заполнена: нужны лицензия с документом, документ личности и селфи.</t>
+  </si>
+  <si>
+    <t>error.api.LICENSE_ALREADY_REGISTERED</t>
+  </si>
+  <si>
+    <t>This license is already linked to another account. If this is a mistake, contact support.</t>
+  </si>
+  <si>
+    <t>Эта лицензия уже привязана к другому аккаунту. Если это ошибка, обратитесь в поддержку.</t>
+  </si>
+  <si>
+    <t>error.api.LICENSE_ALREADY_ADDED</t>
+  </si>
+  <si>
+    <t>A license for this state is already in your request.</t>
+  </si>
+  <si>
+    <t>Лицензия для этого штата уже добавлена в заявку.</t>
+  </si>
+  <si>
+    <t>error.api.ATTORNEY_SUSPENDED</t>
+  </si>
+  <si>
+    <t>Your profile is suspended. Contact support.</t>
+  </si>
+  <si>
+    <t>Профиль приостановлен. Обратитесь в поддержку.</t>
+  </si>
+  <si>
+    <t>notif.verification.in_review</t>
+  </si>
+  <si>
+    <t>Your verification request is being reviewed.</t>
+  </si>
+  <si>
+    <t>Ваша заявка на верификацию взята в работу.</t>
+  </si>
+  <si>
+    <t>notif.verification.needs_more_info</t>
+  </si>
+  <si>
+    <t>The reviewer needs more information: {message}</t>
+  </si>
+  <si>
+    <t>Проверяющему нужна дополнительная информация: {message}</t>
+  </si>
+  <si>
+    <t>notif.verification.approved</t>
+  </si>
+  <si>
+    <t>You're verified. Choose your practice areas to see cases.</t>
+  </si>
+  <si>
+    <t>Верификация пройдена. Выберите практики, чтобы видеть кейсы.</t>
+  </si>
+  <si>
+    <t>notif.verification.approved_partial</t>
+  </si>
+  <si>
+    <t>You're verified, but some licenses were declined. See the status screen for details.</t>
+  </si>
+  <si>
+    <t>Верификация пройдена частично: часть лицензий отклонена. Подробности на экране статуса.</t>
+  </si>
+  <si>
+    <t>notif.verification.rejected</t>
+  </si>
+  <si>
+    <t>Your verification request was declined. See the status screen for the reason and to apply again.</t>
+  </si>
+  <si>
+    <t>Заявка на верификацию отклонена. Причину и повторную подачу смотрите на экране статуса.</t>
+  </si>
+  <si>
+    <t>notif.verification.suspended</t>
+  </si>
+  <si>
+    <t>Your profile has been suspended. Contact support.</t>
+  </si>
+  <si>
+    <t>Ваш профиль приостановлен. Обратитесь в поддержку.</t>
+  </si>
+  <si>
+    <t>notif.verification.restored</t>
+  </si>
+  <si>
+    <t>Your profile has been restored.</t>
+  </si>
+  <si>
+    <t>Ваш профиль восстановлен.</t>
+  </si>
+  <si>
+    <t>verification.reject.license_not_found</t>
+  </si>
+  <si>
+    <t>License not found in the state database</t>
+  </si>
+  <si>
+    <t>Лицензия не найдена в базе штата</t>
+  </si>
+  <si>
+    <t>verification.reject.license_inactive</t>
+  </si>
+  <si>
+    <t>License is inactive</t>
+  </si>
+  <si>
+    <t>Лицензия неактивна</t>
+  </si>
+  <si>
+    <t>verification.reject.name_mismatch</t>
+  </si>
+  <si>
+    <t>Name doesn't match the documents</t>
+  </si>
+  <si>
+    <t>Имя не совпадает с документами</t>
+  </si>
+  <si>
+    <t>verification.reject.document_unreadable</t>
+  </si>
+  <si>
+    <t>Document is unreadable</t>
+  </si>
+  <si>
+    <t>Документ нечитаем</t>
+  </si>
+  <si>
+    <t>verification.reject.document_expired</t>
+  </si>
+  <si>
+    <t>Document has expired</t>
+  </si>
+  <si>
+    <t>Срок действия документа истёк</t>
+  </si>
+  <si>
+    <t>verification.reject.selfie_mismatch</t>
+  </si>
+  <si>
+    <t>Selfie doesn't match the ID photo</t>
+  </si>
+  <si>
+    <t>Селфи не совпадает с фото в документе</t>
+  </si>
+  <si>
+    <t>verification.reject.suspected_fraud</t>
+  </si>
+  <si>
+    <t>Suspected fraud</t>
+  </si>
+  <si>
+    <t>Подозрение на мошенничество</t>
+  </si>
+  <si>
+    <t>verification.reject.incomplete_submission</t>
+  </si>
+  <si>
+    <t>Request is incomplete</t>
+  </si>
+  <si>
+    <t>Заявка заполнена не полностью</t>
+  </si>
+  <si>
+    <t>verification.reject.other</t>
+  </si>
+  <si>
+    <t>Other reason</t>
+  </si>
+  <si>
+    <t>Другая причина</t>
   </si>
 </sst>
 </file>
@@ -3465,7 +3672,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C372"/>
+  <dimension ref="A1:C395"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -7564,6 +7771,259 @@
         <v>1025</v>
       </c>
     </row>
+    <row r="373" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A373" t="s">
+        <v>1026</v>
+      </c>
+      <c r="B373" t="s">
+        <v>1027</v>
+      </c>
+      <c r="C373" t="s">
+        <v>1028</v>
+      </c>
+    </row>
+    <row r="374" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A374" t="s">
+        <v>1029</v>
+      </c>
+      <c r="B374" t="s">
+        <v>1030</v>
+      </c>
+      <c r="C374" t="s">
+        <v>1031</v>
+      </c>
+    </row>
+    <row r="375" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A375" t="s">
+        <v>1032</v>
+      </c>
+      <c r="B375" t="s">
+        <v>1033</v>
+      </c>
+      <c r="C375" t="s">
+        <v>1034</v>
+      </c>
+    </row>
+    <row r="376" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A376" t="s">
+        <v>1035</v>
+      </c>
+      <c r="B376" t="s">
+        <v>1036</v>
+      </c>
+      <c r="C376" t="s">
+        <v>1037</v>
+      </c>
+    </row>
+    <row r="377" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A377" t="s">
+        <v>1038</v>
+      </c>
+      <c r="B377" t="s">
+        <v>1039</v>
+      </c>
+      <c r="C377" t="s">
+        <v>1040</v>
+      </c>
+    </row>
+    <row r="378" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A378" t="s">
+        <v>1041</v>
+      </c>
+      <c r="B378" t="s">
+        <v>1042</v>
+      </c>
+      <c r="C378" t="s">
+        <v>1043</v>
+      </c>
+    </row>
+    <row r="379" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A379" t="s">
+        <v>1044</v>
+      </c>
+      <c r="B379" t="s">
+        <v>1045</v>
+      </c>
+      <c r="C379" t="s">
+        <v>1046</v>
+      </c>
+    </row>
+    <row r="380" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A380" t="s">
+        <v>1047</v>
+      </c>
+      <c r="B380" t="s">
+        <v>1048</v>
+      </c>
+      <c r="C380" t="s">
+        <v>1049</v>
+      </c>
+    </row>
+    <row r="381" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A381" t="s">
+        <v>1050</v>
+      </c>
+      <c r="B381" t="s">
+        <v>1051</v>
+      </c>
+      <c r="C381" t="s">
+        <v>1052</v>
+      </c>
+    </row>
+    <row r="382" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A382" t="s">
+        <v>1053</v>
+      </c>
+      <c r="B382" t="s">
+        <v>1054</v>
+      </c>
+      <c r="C382" t="s">
+        <v>1055</v>
+      </c>
+    </row>
+    <row r="383" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A383" t="s">
+        <v>1056</v>
+      </c>
+      <c r="B383" t="s">
+        <v>1057</v>
+      </c>
+      <c r="C383" t="s">
+        <v>1058</v>
+      </c>
+    </row>
+    <row r="384" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A384" t="s">
+        <v>1059</v>
+      </c>
+      <c r="B384" t="s">
+        <v>1060</v>
+      </c>
+      <c r="C384" t="s">
+        <v>1061</v>
+      </c>
+    </row>
+    <row r="385" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A385" t="s">
+        <v>1062</v>
+      </c>
+      <c r="B385" t="s">
+        <v>1063</v>
+      </c>
+      <c r="C385" t="s">
+        <v>1064</v>
+      </c>
+    </row>
+    <row r="386" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A386" t="s">
+        <v>1065</v>
+      </c>
+      <c r="B386" t="s">
+        <v>1066</v>
+      </c>
+      <c r="C386" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="387" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A387" t="s">
+        <v>1068</v>
+      </c>
+      <c r="B387" t="s">
+        <v>1069</v>
+      </c>
+      <c r="C387" t="s">
+        <v>1070</v>
+      </c>
+    </row>
+    <row r="388" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A388" t="s">
+        <v>1071</v>
+      </c>
+      <c r="B388" t="s">
+        <v>1072</v>
+      </c>
+      <c r="C388" t="s">
+        <v>1073</v>
+      </c>
+    </row>
+    <row r="389" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A389" t="s">
+        <v>1074</v>
+      </c>
+      <c r="B389" t="s">
+        <v>1075</v>
+      </c>
+      <c r="C389" t="s">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="390" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A390" t="s">
+        <v>1077</v>
+      </c>
+      <c r="B390" t="s">
+        <v>1078</v>
+      </c>
+      <c r="C390" t="s">
+        <v>1079</v>
+      </c>
+    </row>
+    <row r="391" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A391" t="s">
+        <v>1080</v>
+      </c>
+      <c r="B391" t="s">
+        <v>1081</v>
+      </c>
+      <c r="C391" t="s">
+        <v>1082</v>
+      </c>
+    </row>
+    <row r="392" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A392" t="s">
+        <v>1083</v>
+      </c>
+      <c r="B392" t="s">
+        <v>1084</v>
+      </c>
+      <c r="C392" t="s">
+        <v>1085</v>
+      </c>
+    </row>
+    <row r="393" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A393" t="s">
+        <v>1086</v>
+      </c>
+      <c r="B393" t="s">
+        <v>1087</v>
+      </c>
+      <c r="C393" t="s">
+        <v>1088</v>
+      </c>
+    </row>
+    <row r="394" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A394" t="s">
+        <v>1089</v>
+      </c>
+      <c r="B394" t="s">
+        <v>1090</v>
+      </c>
+      <c r="C394" t="s">
+        <v>1091</v>
+      </c>
+    </row>
+    <row r="395" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A395" t="s">
+        <v>1092</v>
+      </c>
+      <c r="B395" t="s">
+        <v>1093</v>
+      </c>
+      <c r="C395" t="s">
+        <v>1094</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>

</xml_diff>

<commit_message>
feat: public attorney photo, own case review, mandatory attorney photo (docs/03)
- GET /attorneys/:username returns avatarUrl/avatarUrl256 (clean avatar
  files only, never verification documents); mobile header shows it.
- GET /cases/:caseId/review for the case's client (404 otherwise);
  ReviewDto.editable; mobile review form loads the existing review.
- Attorney photo mandatory (docs/03 §4.1, OQ-012): missing 'photo' ->
  ONBOARDING_INCOMPLETE; mobile guard + required photo row.
- Onboarding actions refused as incomplete reload me and move the user to
  the step owning the missing item, with the localized reason.
- Role screen: an already-set role disables the other card, shows a note,
  Continue moves on without an API call.
- Merge stage 3.9 translation keys; regenerate API contract.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0185gN8jDyiGGwA6x5BUeZUi
</commit_message>
<xml_diff>
--- a/apps/api/prisma/seed/translations_seed.xlsx
+++ b/apps/api/prisma/seed/translations_seed.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1185" uniqueCount="1095">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1605" uniqueCount="1492">
   <si>
     <t>key</t>
   </si>
@@ -3296,6 +3296,1197 @@
   </si>
   <si>
     <t>Другая причина</t>
+  </si>
+  <si>
+    <t>gate.verify.title</t>
+  </si>
+  <si>
+    <t>Complete verification</t>
+  </si>
+  <si>
+    <t>Пройдите верификацию</t>
+  </si>
+  <si>
+    <t>gate.verify.cta</t>
+  </si>
+  <si>
+    <t>Пройти верификацию</t>
+  </si>
+  <si>
+    <t>gate.verify.cases</t>
+  </si>
+  <si>
+    <t>Cases open after LawBid confirms your license. It usually takes 1–2 business days.</t>
+  </si>
+  <si>
+    <t>Кейсы откроются, когда LawBid подтвердит вашу лицензию. Обычно это 1–2 рабочих дня.</t>
+  </si>
+  <si>
+    <t>gate.verify.post</t>
+  </si>
+  <si>
+    <t>Only verified attorneys can post to the feed, so clients always know who they're reading.</t>
+  </si>
+  <si>
+    <t>Публиковать в ленте могут только верифицированные адвокаты — так клиенты всегда знают, кого читают.</t>
+  </si>
+  <si>
+    <t>gate.verify.postTitle</t>
+  </si>
+  <si>
+    <t>Post to feed</t>
+  </si>
+  <si>
+    <t>Пост в ленту</t>
+  </si>
+  <si>
+    <t>practices.title</t>
+  </si>
+  <si>
+    <t>My practices</t>
+  </si>
+  <si>
+    <t>Мои практики</t>
+  </si>
+  <si>
+    <t>practices.intro</t>
+  </si>
+  <si>
+    <t>Pick the specializations you take cases in. Case matching updates right after you save.</t>
+  </si>
+  <si>
+    <t>Выберите специализации, по которым берёте дела. Подбор кейсов обновится сразу после сохранения.</t>
+  </si>
+  <si>
+    <t>practices.search</t>
+  </si>
+  <si>
+    <t>Search practice areas</t>
+  </si>
+  <si>
+    <t>Поиск по практикам</t>
+  </si>
+  <si>
+    <t>practices.selected</t>
+  </si>
+  <si>
+    <t>Selected ({count})</t>
+  </si>
+  <si>
+    <t>Выбрано ({count})</t>
+  </si>
+  <si>
+    <t>practices.selected.none</t>
+  </si>
+  <si>
+    <t>Nothing selected yet.</t>
+  </si>
+  <si>
+    <t>Пока ничего не выбрано.</t>
+  </si>
+  <si>
+    <t>practices.selectAll</t>
+  </si>
+  <si>
+    <t>Select all</t>
+  </si>
+  <si>
+    <t>Выбрать все</t>
+  </si>
+  <si>
+    <t>practices.clearAll</t>
+  </si>
+  <si>
+    <t>Clear all</t>
+  </si>
+  <si>
+    <t>Снять все</t>
+  </si>
+  <si>
+    <t>practices.pickedCount</t>
+  </si>
+  <si>
+    <t>{count} selected</t>
+  </si>
+  <si>
+    <t>Выбрано: {count}</t>
+  </si>
+  <si>
+    <t>practices.remove</t>
+  </si>
+  <si>
+    <t>Remove {name}</t>
+  </si>
+  <si>
+    <t>Убрать {name}</t>
+  </si>
+  <si>
+    <t>practices.save</t>
+  </si>
+  <si>
+    <t>Save</t>
+  </si>
+  <si>
+    <t>Сохранить</t>
+  </si>
+  <si>
+    <t>practices.saved</t>
+  </si>
+  <si>
+    <t>Practices saved.</t>
+  </si>
+  <si>
+    <t>Практики сохранены.</t>
+  </si>
+  <si>
+    <t>practices.noResults</t>
+  </si>
+  <si>
+    <t>No practice areas match your search.</t>
+  </si>
+  <si>
+    <t>По запросу ничего не найдено.</t>
+  </si>
+  <si>
+    <t>practices.emptyTree</t>
+  </si>
+  <si>
+    <t>The practice directory is empty right now. Please try again later.</t>
+  </si>
+  <si>
+    <t>Справочник практик сейчас пуст. Попробуйте позже.</t>
+  </si>
+  <si>
+    <t>practices.error</t>
+  </si>
+  <si>
+    <t>Couldn't load practice areas.</t>
+  </si>
+  <si>
+    <t>Не удалось загрузить практики.</t>
+  </si>
+  <si>
+    <t>practices.locked.title</t>
+  </si>
+  <si>
+    <t>Available after verification</t>
+  </si>
+  <si>
+    <t>Доступно после верификации</t>
+  </si>
+  <si>
+    <t>practices.locked.body</t>
+  </si>
+  <si>
+    <t>Practice areas decide which cases you see, so they open once your license is verified.</t>
+  </si>
+  <si>
+    <t>Практики определяют, какие кейсы вы видите, поэтому они открываются после подтверждения лицензии.</t>
+  </si>
+  <si>
+    <t>profile.tab.title</t>
+  </si>
+  <si>
+    <t>profile.attorney.title</t>
+  </si>
+  <si>
+    <t>profile.attorneyChip</t>
+  </si>
+  <si>
+    <t>profile.avatar.label</t>
+  </si>
+  <si>
+    <t>Profile photo</t>
+  </si>
+  <si>
+    <t>Фото профиля</t>
+  </si>
+  <si>
+    <t>profile.verified.label</t>
+  </si>
+  <si>
+    <t>Verified attorney</t>
+  </si>
+  <si>
+    <t>Верифицированный адвокат</t>
+  </si>
+  <si>
+    <t>profile.counters.posts</t>
+  </si>
+  <si>
+    <t>Posts</t>
+  </si>
+  <si>
+    <t>Посты</t>
+  </si>
+  <si>
+    <t>profile.counters.followers</t>
+  </si>
+  <si>
+    <t>Followers</t>
+  </si>
+  <si>
+    <t>Подписчики</t>
+  </si>
+  <si>
+    <t>profile.counters.following</t>
+  </si>
+  <si>
+    <t>Following</t>
+  </si>
+  <si>
+    <t>Подписки</t>
+  </si>
+  <si>
+    <t>profile.rating.new</t>
+  </si>
+  <si>
+    <t>New — no reviews</t>
+  </si>
+  <si>
+    <t>Новый — без отзывов</t>
+  </si>
+  <si>
+    <t>profile.rating.none</t>
+  </si>
+  <si>
+    <t>—</t>
+  </si>
+  <si>
+    <t>profile.rating.outOf</t>
+  </si>
+  <si>
+    <t>out of 5</t>
+  </si>
+  <si>
+    <t>из 5</t>
+  </si>
+  <si>
+    <t>profile.rating.count.one</t>
+  </si>
+  <si>
+    <t>{count} review</t>
+  </si>
+  <si>
+    <t>{count} отзыв</t>
+  </si>
+  <si>
+    <t>profile.rating.count.few</t>
+  </si>
+  <si>
+    <t>{count} reviews</t>
+  </si>
+  <si>
+    <t>{count} отзыва</t>
+  </si>
+  <si>
+    <t>profile.rating.count.many</t>
+  </si>
+  <si>
+    <t>{count} отзывов</t>
+  </si>
+  <si>
+    <t>profile.rating.count.other</t>
+  </si>
+  <si>
+    <t>profile.section.firm</t>
+  </si>
+  <si>
+    <t>Firm</t>
+  </si>
+  <si>
+    <t>Фирма</t>
+  </si>
+  <si>
+    <t>profile.section.practices</t>
+  </si>
+  <si>
+    <t>Practice areas</t>
+  </si>
+  <si>
+    <t>Практики</t>
+  </si>
+  <si>
+    <t>profile.section.states</t>
+  </si>
+  <si>
+    <t>Licensed in</t>
+  </si>
+  <si>
+    <t>Лицензии в штатах</t>
+  </si>
+  <si>
+    <t>profile.section.languages</t>
+  </si>
+  <si>
+    <t>Languages</t>
+  </si>
+  <si>
+    <t>Языки</t>
+  </si>
+  <si>
+    <t>profile.practices.group</t>
+  </si>
+  <si>
+    <t>{name} · {count}</t>
+  </si>
+  <si>
+    <t>profile.action.edit</t>
+  </si>
+  <si>
+    <t>Edit</t>
+  </si>
+  <si>
+    <t>Редактировать</t>
+  </si>
+  <si>
+    <t>profile.action.share</t>
+  </si>
+  <si>
+    <t>Share</t>
+  </si>
+  <si>
+    <t>Поделиться</t>
+  </si>
+  <si>
+    <t>profile.action.follow</t>
+  </si>
+  <si>
+    <t>Follow</t>
+  </si>
+  <si>
+    <t>Подписаться</t>
+  </si>
+  <si>
+    <t>profile.share.copied</t>
+  </si>
+  <si>
+    <t>Profile link copied.</t>
+  </si>
+  <si>
+    <t>Ссылка на профиль скопирована.</t>
+  </si>
+  <si>
+    <t>profile.tab.posts</t>
+  </si>
+  <si>
+    <t>profile.tab.reviews</t>
+  </si>
+  <si>
+    <t>Reviews</t>
+  </si>
+  <si>
+    <t>Отзывы</t>
+  </si>
+  <si>
+    <t>profile.posts.empty.title</t>
+  </si>
+  <si>
+    <t>No posts yet</t>
+  </si>
+  <si>
+    <t>Постов пока нет</t>
+  </si>
+  <si>
+    <t>profile.posts.empty.self</t>
+  </si>
+  <si>
+    <t>Your posts will appear here.</t>
+  </si>
+  <si>
+    <t>Здесь появятся ваши посты.</t>
+  </si>
+  <si>
+    <t>profile.posts.empty.other</t>
+  </si>
+  <si>
+    <t>This attorney hasn't posted yet.</t>
+  </si>
+  <si>
+    <t>Адвокат пока ничего не публиковал.</t>
+  </si>
+  <si>
+    <t>profile.verifyBanner.body</t>
+  </si>
+  <si>
+    <t>Get the blue check and access to cases.</t>
+  </si>
+  <si>
+    <t>Получите синюю галочку и доступ к кейсам.</t>
+  </si>
+  <si>
+    <t>profile.error</t>
+  </si>
+  <si>
+    <t>Couldn't load the profile.</t>
+  </si>
+  <si>
+    <t>Не удалось загрузить профиль.</t>
+  </si>
+  <si>
+    <t>profile.unavailable.title</t>
+  </si>
+  <si>
+    <t>Profile unavailable</t>
+  </si>
+  <si>
+    <t>Профиль недоступен</t>
+  </si>
+  <si>
+    <t>profile.unavailable.body</t>
+  </si>
+  <si>
+    <t>This profile doesn't exist or can't be shown.</t>
+  </si>
+  <si>
+    <t>Такого профиля нет или его нельзя показать.</t>
+  </si>
+  <si>
+    <t>profile.client.noName</t>
+  </si>
+  <si>
+    <t>Your name</t>
+  </si>
+  <si>
+    <t>Ваше имя</t>
+  </si>
+  <si>
+    <t>profile.client.myCases</t>
+  </si>
+  <si>
+    <t>My cases</t>
+  </si>
+  <si>
+    <t>Мои кейсы</t>
+  </si>
+  <si>
+    <t>profile.client.onlyYou</t>
+  </si>
+  <si>
+    <t>Visible only to you</t>
+  </si>
+  <si>
+    <t>Видно только вам</t>
+  </si>
+  <si>
+    <t>profile.client.noCases</t>
+  </si>
+  <si>
+    <t>You have no cases yet</t>
+  </si>
+  <si>
+    <t>У вас пока нет кейсов</t>
+  </si>
+  <si>
+    <t>profile.client.noCases.body</t>
+  </si>
+  <si>
+    <t>Your profile is private: attorneys and other clients can't see it.</t>
+  </si>
+  <si>
+    <t>Ваш профиль закрыт: его не видят ни адвокаты, ни другие клиенты.</t>
+  </si>
+  <si>
+    <t>profile.edit.title</t>
+  </si>
+  <si>
+    <t>Edit profile</t>
+  </si>
+  <si>
+    <t>Редактирование профиля</t>
+  </si>
+  <si>
+    <t>profile.edit.save</t>
+  </si>
+  <si>
+    <t>profile.edit.saved</t>
+  </si>
+  <si>
+    <t>Profile saved.</t>
+  </si>
+  <si>
+    <t>Профиль сохранён.</t>
+  </si>
+  <si>
+    <t>profile.edit.nameRecheck</t>
+  </si>
+  <si>
+    <t>Changing your name sends your profile for a quick re-check so it matches your documents.</t>
+  </si>
+  <si>
+    <t>После смены имени профиль уйдёт на короткую повторную проверку, чтобы имя совпадало с документами.</t>
+  </si>
+  <si>
+    <t>profile.edit.section.practice</t>
+  </si>
+  <si>
+    <t>Practice</t>
+  </si>
+  <si>
+    <t>Практика</t>
+  </si>
+  <si>
+    <t>profile.edit.section.licenses</t>
+  </si>
+  <si>
+    <t>Licenses</t>
+  </si>
+  <si>
+    <t>Лицензии</t>
+  </si>
+  <si>
+    <t>profile.license.pending</t>
+  </si>
+  <si>
+    <t>Under review</t>
+  </si>
+  <si>
+    <t>На проверке</t>
+  </si>
+  <si>
+    <t>profile.license.verified</t>
+  </si>
+  <si>
+    <t>Подтверждена</t>
+  </si>
+  <si>
+    <t>profile.license.rejected</t>
+  </si>
+  <si>
+    <t>Rejected</t>
+  </si>
+  <si>
+    <t>Отклонена</t>
+  </si>
+  <si>
+    <t>profile.license.expired</t>
+  </si>
+  <si>
+    <t>Expired</t>
+  </si>
+  <si>
+    <t>Истекла</t>
+  </si>
+  <si>
+    <t>profile.license.suspended</t>
+  </si>
+  <si>
+    <t>Suspended</t>
+  </si>
+  <si>
+    <t>Приостановлена</t>
+  </si>
+  <si>
+    <t>profile.license.unknown</t>
+  </si>
+  <si>
+    <t>Unknown</t>
+  </si>
+  <si>
+    <t>Неизвестно</t>
+  </si>
+  <si>
+    <t>profile.username.label</t>
+  </si>
+  <si>
+    <t>Username</t>
+  </si>
+  <si>
+    <t>Имя пользователя</t>
+  </si>
+  <si>
+    <t>profile.username.hint</t>
+  </si>
+  <si>
+    <t>3–30 letters, digits, "_" or ".". You can change it once every 30 days.</t>
+  </si>
+  <si>
+    <t>3–30 символов: латиница, цифры, «_» или «.». Менять можно раз в 30 дней.</t>
+  </si>
+  <si>
+    <t>profile.username.cooldown</t>
+  </si>
+  <si>
+    <t>You can change your @username again on {date}.</t>
+  </si>
+  <si>
+    <t>Сменить @username снова можно {date}.</t>
+  </si>
+  <si>
+    <t>profile.username.checking</t>
+  </si>
+  <si>
+    <t>Checking…</t>
+  </si>
+  <si>
+    <t>Проверяем…</t>
+  </si>
+  <si>
+    <t>profile.username.available</t>
+  </si>
+  <si>
+    <t>This @username is available.</t>
+  </si>
+  <si>
+    <t>Этот @username свободен.</t>
+  </si>
+  <si>
+    <t>profile.username.invalid</t>
+  </si>
+  <si>
+    <t>Use 3–30 latin letters, digits, "_" or "."; not at the start or end, no "..".</t>
+  </si>
+  <si>
+    <t>3–30 символов: латиница, цифры, «_» или «.»; не в начале и не в конце, без «..».</t>
+  </si>
+  <si>
+    <t>profile.username.checkFailed</t>
+  </si>
+  <si>
+    <t>Couldn't check availability. We'll check when you save.</t>
+  </si>
+  <si>
+    <t>Не удалось проверить. Проверим при сохранении.</t>
+  </si>
+  <si>
+    <t>profile.photo.label</t>
+  </si>
+  <si>
+    <t>profile.photo.hint</t>
+  </si>
+  <si>
+    <t>A clear business photo. JPEG, PNG or HEIC, up to 5 MB.</t>
+  </si>
+  <si>
+    <t>Чёткое деловое фото. JPEG, PNG или HEIC, до 5 МБ.</t>
+  </si>
+  <si>
+    <t>profile.photo.add</t>
+  </si>
+  <si>
+    <t>Add photo</t>
+  </si>
+  <si>
+    <t>Добавить фото</t>
+  </si>
+  <si>
+    <t>profile.photo.change</t>
+  </si>
+  <si>
+    <t>Change photo</t>
+  </si>
+  <si>
+    <t>Изменить фото</t>
+  </si>
+  <si>
+    <t>profile.photo.camera</t>
+  </si>
+  <si>
+    <t>Take a photo</t>
+  </si>
+  <si>
+    <t>Сделать фото</t>
+  </si>
+  <si>
+    <t>profile.photo.gallery</t>
+  </si>
+  <si>
+    <t>Choose from library</t>
+  </si>
+  <si>
+    <t>Выбрать из галереи</t>
+  </si>
+  <si>
+    <t>profile.photo.preparing</t>
+  </si>
+  <si>
+    <t>Preparing…</t>
+  </si>
+  <si>
+    <t>Подготовка…</t>
+  </si>
+  <si>
+    <t>profile.photo.uploading</t>
+  </si>
+  <si>
+    <t>Uploading… {percent}%</t>
+  </si>
+  <si>
+    <t>Загрузка… {percent}%</t>
+  </si>
+  <si>
+    <t>profile.photo.checking</t>
+  </si>
+  <si>
+    <t>Checking the photo…</t>
+  </si>
+  <si>
+    <t>Проверяем фото…</t>
+  </si>
+  <si>
+    <t>profile.photo.done</t>
+  </si>
+  <si>
+    <t>Photo updated.</t>
+  </si>
+  <si>
+    <t>Фото обновлено.</t>
+  </si>
+  <si>
+    <t>profile.photo.pickFailed</t>
+  </si>
+  <si>
+    <t>Couldn't open the photo. Please try another one.</t>
+  </si>
+  <si>
+    <t>Не удалось открыть фото. Попробуйте другое.</t>
+  </si>
+  <si>
+    <t>contacts.title</t>
+  </si>
+  <si>
+    <t>My contacts</t>
+  </si>
+  <si>
+    <t>Мои контакты</t>
+  </si>
+  <si>
+    <t>contacts.section.confirmed</t>
+  </si>
+  <si>
+    <t>Confirmed contacts</t>
+  </si>
+  <si>
+    <t>Подтверждённые контакты</t>
+  </si>
+  <si>
+    <t>contacts.section.preferences</t>
+  </si>
+  <si>
+    <t>How attorneys can reach you</t>
+  </si>
+  <si>
+    <t>Как с вами связаться</t>
+  </si>
+  <si>
+    <t>contacts.prefs.saved</t>
+  </si>
+  <si>
+    <t>Contact preferences saved.</t>
+  </si>
+  <si>
+    <t>Предпочтения связи сохранены.</t>
+  </si>
+  <si>
+    <t>contacts.prefs.error</t>
+  </si>
+  <si>
+    <t>Couldn't load your contact preferences.</t>
+  </si>
+  <si>
+    <t>Не удалось загрузить предпочтения связи.</t>
+  </si>
+  <si>
+    <t>reviews.author.anonymous</t>
+  </si>
+  <si>
+    <t>LawBid client</t>
+  </si>
+  <si>
+    <t>Клиент LawBid</t>
+  </si>
+  <si>
+    <t>reviews.edited</t>
+  </si>
+  <si>
+    <t>Edited</t>
+  </si>
+  <si>
+    <t>Изменено</t>
+  </si>
+  <si>
+    <t>reviews.stars.label</t>
+  </si>
+  <si>
+    <t>{rating} out of 5 stars</t>
+  </si>
+  <si>
+    <t>{rating} из 5 звёзд</t>
+  </si>
+  <si>
+    <t>reviews.average.label</t>
+  </si>
+  <si>
+    <t>Rating {rating} out of 5</t>
+  </si>
+  <si>
+    <t>Рейтинг {rating} из 5</t>
+  </si>
+  <si>
+    <t>reviews.distribution.row</t>
+  </si>
+  <si>
+    <t>{stars} stars: {count}</t>
+  </si>
+  <si>
+    <t>{stars} звёзд: {count}</t>
+  </si>
+  <si>
+    <t>reviews.end</t>
+  </si>
+  <si>
+    <t>That's all the reviews</t>
+  </si>
+  <si>
+    <t>Это все отзывы</t>
+  </si>
+  <si>
+    <t>reviews.error</t>
+  </si>
+  <si>
+    <t>Couldn't load reviews.</t>
+  </si>
+  <si>
+    <t>Не удалось загрузить отзывы.</t>
+  </si>
+  <si>
+    <t>reviews.empty.self</t>
+  </si>
+  <si>
+    <t>When clients rate your work after a closed case, reviews will appear here.</t>
+  </si>
+  <si>
+    <t>Когда клиенты оценят вашу работу по закрытому кейсу, отзывы появятся здесь.</t>
+  </si>
+  <si>
+    <t>reviews.empty.other</t>
+  </si>
+  <si>
+    <t>This attorney has no reviews yet.</t>
+  </si>
+  <si>
+    <t>У этого адвоката пока нет отзывов.</t>
+  </si>
+  <si>
+    <t>reviews.report.action</t>
+  </si>
+  <si>
+    <t>Report review</t>
+  </si>
+  <si>
+    <t>Пожаловаться на отзыв</t>
+  </si>
+  <si>
+    <t>reviews.report.title</t>
+  </si>
+  <si>
+    <t>Why are you reporting this review?</t>
+  </si>
+  <si>
+    <t>Почему вы жалуетесь на отзыв?</t>
+  </si>
+  <si>
+    <t>reviews.report.sent</t>
+  </si>
+  <si>
+    <t>Thanks. Our moderators will review it.</t>
+  </si>
+  <si>
+    <t>Спасибо. Модераторы рассмотрят жалобу.</t>
+  </si>
+  <si>
+    <t>reviews.report.reason.spam</t>
+  </si>
+  <si>
+    <t>Spam</t>
+  </si>
+  <si>
+    <t>Спам</t>
+  </si>
+  <si>
+    <t>reviews.report.reason.abuse</t>
+  </si>
+  <si>
+    <t>Abuse or harassment</t>
+  </si>
+  <si>
+    <t>Оскорбления или травля</t>
+  </si>
+  <si>
+    <t>reviews.report.reason.misinformation</t>
+  </si>
+  <si>
+    <t>False information</t>
+  </si>
+  <si>
+    <t>Ложная информация</t>
+  </si>
+  <si>
+    <t>reviews.report.reason.impersonation</t>
+  </si>
+  <si>
+    <t>Not a real client</t>
+  </si>
+  <si>
+    <t>Не настоящий клиент</t>
+  </si>
+  <si>
+    <t>reviews.report.reason.inappropriate</t>
+  </si>
+  <si>
+    <t>Inappropriate content</t>
+  </si>
+  <si>
+    <t>Неуместное содержание</t>
+  </si>
+  <si>
+    <t>reviews.report.reason.other</t>
+  </si>
+  <si>
+    <t>Other</t>
+  </si>
+  <si>
+    <t>Другое</t>
+  </si>
+  <si>
+    <t>reviews.form.title</t>
+  </si>
+  <si>
+    <t>Rate your attorney</t>
+  </si>
+  <si>
+    <t>Оцените адвоката</t>
+  </si>
+  <si>
+    <t>reviews.form.titleYours</t>
+  </si>
+  <si>
+    <t>Your review</t>
+  </si>
+  <si>
+    <t>Ваш отзыв</t>
+  </si>
+  <si>
+    <t>reviews.form.question</t>
+  </si>
+  <si>
+    <t>How did your attorney handle the case?</t>
+  </si>
+  <si>
+    <t>Как адвокат вёл ваше дело?</t>
+  </si>
+  <si>
+    <t>reviews.form.tapToRate</t>
+  </si>
+  <si>
+    <t>Tap a star to rate</t>
+  </si>
+  <si>
+    <t>Нажмите на звезду, чтобы оценить</t>
+  </si>
+  <si>
+    <t>reviews.form.ratingRequired</t>
+  </si>
+  <si>
+    <t>Please choose a rating</t>
+  </si>
+  <si>
+    <t>Выберите оценку</t>
+  </si>
+  <si>
+    <t>reviews.form.rating.1</t>
+  </si>
+  <si>
+    <t>Poor</t>
+  </si>
+  <si>
+    <t>Плохо</t>
+  </si>
+  <si>
+    <t>reviews.form.rating.2</t>
+  </si>
+  <si>
+    <t>Fair</t>
+  </si>
+  <si>
+    <t>Так себе</t>
+  </si>
+  <si>
+    <t>reviews.form.rating.3</t>
+  </si>
+  <si>
+    <t>Good</t>
+  </si>
+  <si>
+    <t>Хорошо</t>
+  </si>
+  <si>
+    <t>reviews.form.rating.4</t>
+  </si>
+  <si>
+    <t>Very good</t>
+  </si>
+  <si>
+    <t>Очень хорошо</t>
+  </si>
+  <si>
+    <t>reviews.form.rating.5</t>
+  </si>
+  <si>
+    <t>Excellent</t>
+  </si>
+  <si>
+    <t>Отлично</t>
+  </si>
+  <si>
+    <t>reviews.form.body</t>
+  </si>
+  <si>
+    <t>reviews.form.bodyHint</t>
+  </si>
+  <si>
+    <t>What went well, what could be better</t>
+  </si>
+  <si>
+    <t>Что понравилось, что можно улучшить</t>
+  </si>
+  <si>
+    <t>reviews.form.notice</t>
+  </si>
+  <si>
+    <t>A review can't be deleted. You can edit it within 14 days.</t>
+  </si>
+  <si>
+    <t>Отзыв нельзя удалить, его можно изменить в течение 14 дней.</t>
+  </si>
+  <si>
+    <t>reviews.form.submit</t>
+  </si>
+  <si>
+    <t>Publish review</t>
+  </si>
+  <si>
+    <t>Опубликовать отзыв</t>
+  </si>
+  <si>
+    <t>reviews.form.saveEdit</t>
+  </si>
+  <si>
+    <t>Save changes</t>
+  </si>
+  <si>
+    <t>Сохранить изменения</t>
+  </si>
+  <si>
+    <t>reviews.form.published</t>
+  </si>
+  <si>
+    <t>Review published.</t>
+  </si>
+  <si>
+    <t>Отзыв опубликован.</t>
+  </si>
+  <si>
+    <t>reviews.form.updated</t>
+  </si>
+  <si>
+    <t>Review updated.</t>
+  </si>
+  <si>
+    <t>Отзыв изменён.</t>
+  </si>
+  <si>
+    <t>reviews.form.publishedHeading</t>
+  </si>
+  <si>
+    <t>Your review is published</t>
+  </si>
+  <si>
+    <t>Ваш отзыв опубликован</t>
+  </si>
+  <si>
+    <t>reviews.form.previewHint</t>
+  </si>
+  <si>
+    <t>This is how others see it — your first name and last initial only.</t>
+  </si>
+  <si>
+    <t>Так его видят другие — только имя и первая буква фамилии.</t>
+  </si>
+  <si>
+    <t>reviews.form.edit</t>
+  </si>
+  <si>
+    <t>Edit review</t>
+  </si>
+  <si>
+    <t>Изменить отзыв</t>
+  </si>
+  <si>
+    <t>reviews.form.editableUntil</t>
+  </si>
+  <si>
+    <t>You can edit it until {date}.</t>
+  </si>
+  <si>
+    <t>Изменить можно до {date}.</t>
+  </si>
+  <si>
+    <t>reviews.form.locked</t>
+  </si>
+  <si>
+    <t>The 14-day editing window has ended, so this review can no longer be changed.</t>
+  </si>
+  <si>
+    <t>14 дней на изменение прошли, отзыв больше нельзя изменить.</t>
+  </si>
+  <si>
+    <t>reviews.placeholder.entry</t>
+  </si>
+  <si>
+    <t>Leave a review for a closed case</t>
+  </si>
+  <si>
+    <t>Оставить отзыв по закрытому кейсу</t>
+  </si>
+  <si>
+    <t>reviews.placeholder.body</t>
+  </si>
+  <si>
+    <t>Preview build: closed cases arrive with the cases module. Enter the case ID to open the review form.</t>
+  </si>
+  <si>
+    <t>Тестовая сборка: закрытые кейсы появятся вместе с модулем кейсов. Введите ID кейса, чтобы открыть форму отзыва.</t>
+  </si>
+  <si>
+    <t>reviews.placeholder.caseId</t>
+  </si>
+  <si>
+    <t>Case ID</t>
+  </si>
+  <si>
+    <t>ID кейса</t>
+  </si>
+  <si>
+    <t>error.default.title</t>
+  </si>
+  <si>
+    <t>onboarding.profile.error.photoRequired</t>
+  </si>
+  <si>
+    <t>Add a photo — it is required for attorneys.</t>
+  </si>
+  <si>
+    <t>Добавьте фото — для адвоката оно обязательно.</t>
+  </si>
+  <si>
+    <t>onboarding.role.locked</t>
+  </si>
+  <si>
+    <t>Your role is already set and can't be changed.</t>
+  </si>
+  <si>
+    <t>Роль уже выбрана и не может быть изменена.</t>
   </si>
 </sst>
 </file>
@@ -3672,7 +4863,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C395"/>
+  <dimension ref="A1:C535"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -8024,6 +9215,1546 @@
         <v>1094</v>
       </c>
     </row>
+    <row r="396" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A396" t="s">
+        <v>1095</v>
+      </c>
+      <c r="B396" t="s">
+        <v>1096</v>
+      </c>
+      <c r="C396" t="s">
+        <v>1097</v>
+      </c>
+    </row>
+    <row r="397" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A397" t="s">
+        <v>1098</v>
+      </c>
+      <c r="B397" t="s">
+        <v>1096</v>
+      </c>
+      <c r="C397" t="s">
+        <v>1099</v>
+      </c>
+    </row>
+    <row r="398" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A398" t="s">
+        <v>1100</v>
+      </c>
+      <c r="B398" t="s">
+        <v>1101</v>
+      </c>
+      <c r="C398" t="s">
+        <v>1102</v>
+      </c>
+    </row>
+    <row r="399" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A399" t="s">
+        <v>1103</v>
+      </c>
+      <c r="B399" t="s">
+        <v>1104</v>
+      </c>
+      <c r="C399" t="s">
+        <v>1105</v>
+      </c>
+    </row>
+    <row r="400" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A400" t="s">
+        <v>1106</v>
+      </c>
+      <c r="B400" t="s">
+        <v>1107</v>
+      </c>
+      <c r="C400" t="s">
+        <v>1108</v>
+      </c>
+    </row>
+    <row r="401" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A401" t="s">
+        <v>1109</v>
+      </c>
+      <c r="B401" t="s">
+        <v>1110</v>
+      </c>
+      <c r="C401" t="s">
+        <v>1111</v>
+      </c>
+    </row>
+    <row r="402" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A402" t="s">
+        <v>1112</v>
+      </c>
+      <c r="B402" t="s">
+        <v>1113</v>
+      </c>
+      <c r="C402" t="s">
+        <v>1114</v>
+      </c>
+    </row>
+    <row r="403" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A403" t="s">
+        <v>1115</v>
+      </c>
+      <c r="B403" t="s">
+        <v>1116</v>
+      </c>
+      <c r="C403" t="s">
+        <v>1117</v>
+      </c>
+    </row>
+    <row r="404" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A404" t="s">
+        <v>1118</v>
+      </c>
+      <c r="B404" t="s">
+        <v>1119</v>
+      </c>
+      <c r="C404" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="405" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A405" t="s">
+        <v>1121</v>
+      </c>
+      <c r="B405" t="s">
+        <v>1122</v>
+      </c>
+      <c r="C405" t="s">
+        <v>1123</v>
+      </c>
+    </row>
+    <row r="406" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A406" t="s">
+        <v>1124</v>
+      </c>
+      <c r="B406" t="s">
+        <v>1125</v>
+      </c>
+      <c r="C406" t="s">
+        <v>1126</v>
+      </c>
+    </row>
+    <row r="407" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A407" t="s">
+        <v>1127</v>
+      </c>
+      <c r="B407" t="s">
+        <v>1128</v>
+      </c>
+      <c r="C407" t="s">
+        <v>1129</v>
+      </c>
+    </row>
+    <row r="408" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A408" t="s">
+        <v>1130</v>
+      </c>
+      <c r="B408" t="s">
+        <v>1131</v>
+      </c>
+      <c r="C408" t="s">
+        <v>1132</v>
+      </c>
+    </row>
+    <row r="409" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A409" t="s">
+        <v>1133</v>
+      </c>
+      <c r="B409" t="s">
+        <v>1134</v>
+      </c>
+      <c r="C409" t="s">
+        <v>1135</v>
+      </c>
+    </row>
+    <row r="410" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A410" t="s">
+        <v>1136</v>
+      </c>
+      <c r="B410" t="s">
+        <v>1137</v>
+      </c>
+      <c r="C410" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="411" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A411" t="s">
+        <v>1139</v>
+      </c>
+      <c r="B411" t="s">
+        <v>1140</v>
+      </c>
+      <c r="C411" t="s">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="412" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A412" t="s">
+        <v>1142</v>
+      </c>
+      <c r="B412" t="s">
+        <v>1143</v>
+      </c>
+      <c r="C412" t="s">
+        <v>1144</v>
+      </c>
+    </row>
+    <row r="413" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A413" t="s">
+        <v>1145</v>
+      </c>
+      <c r="B413" t="s">
+        <v>1146</v>
+      </c>
+      <c r="C413" t="s">
+        <v>1147</v>
+      </c>
+    </row>
+    <row r="414" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A414" t="s">
+        <v>1148</v>
+      </c>
+      <c r="B414" t="s">
+        <v>1149</v>
+      </c>
+      <c r="C414" t="s">
+        <v>1150</v>
+      </c>
+    </row>
+    <row r="415" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A415" t="s">
+        <v>1151</v>
+      </c>
+      <c r="B415" t="s">
+        <v>1152</v>
+      </c>
+      <c r="C415" t="s">
+        <v>1153</v>
+      </c>
+    </row>
+    <row r="416" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A416" t="s">
+        <v>1154</v>
+      </c>
+      <c r="B416" t="s">
+        <v>1155</v>
+      </c>
+      <c r="C416" t="s">
+        <v>1156</v>
+      </c>
+    </row>
+    <row r="417" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A417" t="s">
+        <v>1157</v>
+      </c>
+      <c r="B417" t="s">
+        <v>253</v>
+      </c>
+      <c r="C417" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="418" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A418" t="s">
+        <v>1158</v>
+      </c>
+      <c r="B418" t="s">
+        <v>264</v>
+      </c>
+      <c r="C418" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="419" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A419" t="s">
+        <v>1159</v>
+      </c>
+      <c r="B419" t="s">
+        <v>264</v>
+      </c>
+      <c r="C419" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="420" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A420" t="s">
+        <v>1160</v>
+      </c>
+      <c r="B420" t="s">
+        <v>1161</v>
+      </c>
+      <c r="C420" t="s">
+        <v>1162</v>
+      </c>
+    </row>
+    <row r="421" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A421" t="s">
+        <v>1163</v>
+      </c>
+      <c r="B421" t="s">
+        <v>1164</v>
+      </c>
+      <c r="C421" t="s">
+        <v>1165</v>
+      </c>
+    </row>
+    <row r="422" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A422" t="s">
+        <v>1166</v>
+      </c>
+      <c r="B422" t="s">
+        <v>1167</v>
+      </c>
+      <c r="C422" t="s">
+        <v>1168</v>
+      </c>
+    </row>
+    <row r="423" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A423" t="s">
+        <v>1169</v>
+      </c>
+      <c r="B423" t="s">
+        <v>1170</v>
+      </c>
+      <c r="C423" t="s">
+        <v>1171</v>
+      </c>
+    </row>
+    <row r="424" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A424" t="s">
+        <v>1172</v>
+      </c>
+      <c r="B424" t="s">
+        <v>1173</v>
+      </c>
+      <c r="C424" t="s">
+        <v>1174</v>
+      </c>
+    </row>
+    <row r="425" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A425" t="s">
+        <v>1175</v>
+      </c>
+      <c r="B425" t="s">
+        <v>1176</v>
+      </c>
+      <c r="C425" t="s">
+        <v>1177</v>
+      </c>
+    </row>
+    <row r="426" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A426" t="s">
+        <v>1178</v>
+      </c>
+      <c r="B426" t="s">
+        <v>1179</v>
+      </c>
+      <c r="C426" t="s">
+        <v>1179</v>
+      </c>
+    </row>
+    <row r="427" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A427" t="s">
+        <v>1180</v>
+      </c>
+      <c r="B427" t="s">
+        <v>1181</v>
+      </c>
+      <c r="C427" t="s">
+        <v>1182</v>
+      </c>
+    </row>
+    <row r="428" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A428" t="s">
+        <v>1183</v>
+      </c>
+      <c r="B428" t="s">
+        <v>1184</v>
+      </c>
+      <c r="C428" t="s">
+        <v>1185</v>
+      </c>
+    </row>
+    <row r="429" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A429" t="s">
+        <v>1186</v>
+      </c>
+      <c r="B429" t="s">
+        <v>1187</v>
+      </c>
+      <c r="C429" t="s">
+        <v>1188</v>
+      </c>
+    </row>
+    <row r="430" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A430" t="s">
+        <v>1189</v>
+      </c>
+      <c r="B430" t="s">
+        <v>1187</v>
+      </c>
+      <c r="C430" t="s">
+        <v>1190</v>
+      </c>
+    </row>
+    <row r="431" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A431" t="s">
+        <v>1191</v>
+      </c>
+      <c r="B431" t="s">
+        <v>1187</v>
+      </c>
+      <c r="C431" t="s">
+        <v>1188</v>
+      </c>
+    </row>
+    <row r="432" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A432" t="s">
+        <v>1192</v>
+      </c>
+      <c r="B432" t="s">
+        <v>1193</v>
+      </c>
+      <c r="C432" t="s">
+        <v>1194</v>
+      </c>
+    </row>
+    <row r="433" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A433" t="s">
+        <v>1195</v>
+      </c>
+      <c r="B433" t="s">
+        <v>1196</v>
+      </c>
+      <c r="C433" t="s">
+        <v>1197</v>
+      </c>
+    </row>
+    <row r="434" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A434" t="s">
+        <v>1198</v>
+      </c>
+      <c r="B434" t="s">
+        <v>1199</v>
+      </c>
+      <c r="C434" t="s">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="435" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A435" t="s">
+        <v>1201</v>
+      </c>
+      <c r="B435" t="s">
+        <v>1202</v>
+      </c>
+      <c r="C435" t="s">
+        <v>1203</v>
+      </c>
+    </row>
+    <row r="436" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A436" t="s">
+        <v>1204</v>
+      </c>
+      <c r="B436" t="s">
+        <v>1205</v>
+      </c>
+      <c r="C436" t="s">
+        <v>1205</v>
+      </c>
+    </row>
+    <row r="437" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A437" t="s">
+        <v>1206</v>
+      </c>
+      <c r="B437" t="s">
+        <v>1207</v>
+      </c>
+      <c r="C437" t="s">
+        <v>1208</v>
+      </c>
+    </row>
+    <row r="438" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A438" t="s">
+        <v>1209</v>
+      </c>
+      <c r="B438" t="s">
+        <v>1210</v>
+      </c>
+      <c r="C438" t="s">
+        <v>1211</v>
+      </c>
+    </row>
+    <row r="439" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A439" t="s">
+        <v>1212</v>
+      </c>
+      <c r="B439" t="s">
+        <v>1213</v>
+      </c>
+      <c r="C439" t="s">
+        <v>1214</v>
+      </c>
+    </row>
+    <row r="440" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A440" t="s">
+        <v>1215</v>
+      </c>
+      <c r="B440" t="s">
+        <v>1216</v>
+      </c>
+      <c r="C440" t="s">
+        <v>1217</v>
+      </c>
+    </row>
+    <row r="441" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A441" t="s">
+        <v>1218</v>
+      </c>
+      <c r="B441" t="s">
+        <v>1167</v>
+      </c>
+      <c r="C441" t="s">
+        <v>1168</v>
+      </c>
+    </row>
+    <row r="442" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A442" t="s">
+        <v>1219</v>
+      </c>
+      <c r="B442" t="s">
+        <v>1220</v>
+      </c>
+      <c r="C442" t="s">
+        <v>1221</v>
+      </c>
+    </row>
+    <row r="443" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A443" t="s">
+        <v>1222</v>
+      </c>
+      <c r="B443" t="s">
+        <v>1223</v>
+      </c>
+      <c r="C443" t="s">
+        <v>1224</v>
+      </c>
+    </row>
+    <row r="444" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A444" t="s">
+        <v>1225</v>
+      </c>
+      <c r="B444" t="s">
+        <v>1226</v>
+      </c>
+      <c r="C444" t="s">
+        <v>1227</v>
+      </c>
+    </row>
+    <row r="445" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A445" t="s">
+        <v>1228</v>
+      </c>
+      <c r="B445" t="s">
+        <v>1229</v>
+      </c>
+      <c r="C445" t="s">
+        <v>1230</v>
+      </c>
+    </row>
+    <row r="446" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A446" t="s">
+        <v>1231</v>
+      </c>
+      <c r="B446" t="s">
+        <v>1232</v>
+      </c>
+      <c r="C446" t="s">
+        <v>1233</v>
+      </c>
+    </row>
+    <row r="447" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A447" t="s">
+        <v>1234</v>
+      </c>
+      <c r="B447" t="s">
+        <v>1235</v>
+      </c>
+      <c r="C447" t="s">
+        <v>1236</v>
+      </c>
+    </row>
+    <row r="448" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A448" t="s">
+        <v>1237</v>
+      </c>
+      <c r="B448" t="s">
+        <v>1238</v>
+      </c>
+      <c r="C448" t="s">
+        <v>1239</v>
+      </c>
+    </row>
+    <row r="449" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A449" t="s">
+        <v>1240</v>
+      </c>
+      <c r="B449" t="s">
+        <v>1241</v>
+      </c>
+      <c r="C449" t="s">
+        <v>1242</v>
+      </c>
+    </row>
+    <row r="450" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A450" t="s">
+        <v>1243</v>
+      </c>
+      <c r="B450" t="s">
+        <v>1244</v>
+      </c>
+      <c r="C450" t="s">
+        <v>1245</v>
+      </c>
+    </row>
+    <row r="451" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A451" t="s">
+        <v>1246</v>
+      </c>
+      <c r="B451" t="s">
+        <v>1247</v>
+      </c>
+      <c r="C451" t="s">
+        <v>1248</v>
+      </c>
+    </row>
+    <row r="452" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A452" t="s">
+        <v>1249</v>
+      </c>
+      <c r="B452" t="s">
+        <v>1250</v>
+      </c>
+      <c r="C452" t="s">
+        <v>1251</v>
+      </c>
+    </row>
+    <row r="453" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A453" t="s">
+        <v>1252</v>
+      </c>
+      <c r="B453" t="s">
+        <v>1253</v>
+      </c>
+      <c r="C453" t="s">
+        <v>1254</v>
+      </c>
+    </row>
+    <row r="454" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A454" t="s">
+        <v>1255</v>
+      </c>
+      <c r="B454" t="s">
+        <v>1256</v>
+      </c>
+      <c r="C454" t="s">
+        <v>1257</v>
+      </c>
+    </row>
+    <row r="455" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A455" t="s">
+        <v>1258</v>
+      </c>
+      <c r="B455" t="s">
+        <v>1259</v>
+      </c>
+      <c r="C455" t="s">
+        <v>1260</v>
+      </c>
+    </row>
+    <row r="456" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A456" t="s">
+        <v>1261</v>
+      </c>
+      <c r="B456" t="s">
+        <v>1137</v>
+      </c>
+      <c r="C456" t="s">
+        <v>1138</v>
+      </c>
+    </row>
+    <row r="457" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A457" t="s">
+        <v>1262</v>
+      </c>
+      <c r="B457" t="s">
+        <v>1263</v>
+      </c>
+      <c r="C457" t="s">
+        <v>1264</v>
+      </c>
+    </row>
+    <row r="458" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A458" t="s">
+        <v>1265</v>
+      </c>
+      <c r="B458" t="s">
+        <v>1266</v>
+      </c>
+      <c r="C458" t="s">
+        <v>1267</v>
+      </c>
+    </row>
+    <row r="459" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A459" t="s">
+        <v>1268</v>
+      </c>
+      <c r="B459" t="s">
+        <v>1269</v>
+      </c>
+      <c r="C459" t="s">
+        <v>1270</v>
+      </c>
+    </row>
+    <row r="460" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A460" t="s">
+        <v>1271</v>
+      </c>
+      <c r="B460" t="s">
+        <v>1272</v>
+      </c>
+      <c r="C460" t="s">
+        <v>1273</v>
+      </c>
+    </row>
+    <row r="461" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A461" t="s">
+        <v>1274</v>
+      </c>
+      <c r="B461" t="s">
+        <v>1275</v>
+      </c>
+      <c r="C461" t="s">
+        <v>1276</v>
+      </c>
+    </row>
+    <row r="462" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A462" t="s">
+        <v>1277</v>
+      </c>
+      <c r="B462" t="s">
+        <v>543</v>
+      </c>
+      <c r="C462" t="s">
+        <v>1278</v>
+      </c>
+    </row>
+    <row r="463" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A463" t="s">
+        <v>1279</v>
+      </c>
+      <c r="B463" t="s">
+        <v>1280</v>
+      </c>
+      <c r="C463" t="s">
+        <v>1281</v>
+      </c>
+    </row>
+    <row r="464" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A464" t="s">
+        <v>1282</v>
+      </c>
+      <c r="B464" t="s">
+        <v>1283</v>
+      </c>
+      <c r="C464" t="s">
+        <v>1284</v>
+      </c>
+    </row>
+    <row r="465" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A465" t="s">
+        <v>1285</v>
+      </c>
+      <c r="B465" t="s">
+        <v>1286</v>
+      </c>
+      <c r="C465" t="s">
+        <v>1287</v>
+      </c>
+    </row>
+    <row r="466" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A466" t="s">
+        <v>1288</v>
+      </c>
+      <c r="B466" t="s">
+        <v>1289</v>
+      </c>
+      <c r="C466" t="s">
+        <v>1290</v>
+      </c>
+    </row>
+    <row r="467" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A467" t="s">
+        <v>1291</v>
+      </c>
+      <c r="B467" t="s">
+        <v>1292</v>
+      </c>
+      <c r="C467" t="s">
+        <v>1293</v>
+      </c>
+    </row>
+    <row r="468" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A468" t="s">
+        <v>1294</v>
+      </c>
+      <c r="B468" t="s">
+        <v>1295</v>
+      </c>
+      <c r="C468" t="s">
+        <v>1296</v>
+      </c>
+    </row>
+    <row r="469" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A469" t="s">
+        <v>1297</v>
+      </c>
+      <c r="B469" t="s">
+        <v>1298</v>
+      </c>
+      <c r="C469" t="s">
+        <v>1299</v>
+      </c>
+    </row>
+    <row r="470" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A470" t="s">
+        <v>1300</v>
+      </c>
+      <c r="B470" t="s">
+        <v>1301</v>
+      </c>
+      <c r="C470" t="s">
+        <v>1302</v>
+      </c>
+    </row>
+    <row r="471" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A471" t="s">
+        <v>1303</v>
+      </c>
+      <c r="B471" t="s">
+        <v>1304</v>
+      </c>
+      <c r="C471" t="s">
+        <v>1305</v>
+      </c>
+    </row>
+    <row r="472" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A472" t="s">
+        <v>1306</v>
+      </c>
+      <c r="B472" t="s">
+        <v>1307</v>
+      </c>
+      <c r="C472" t="s">
+        <v>1308</v>
+      </c>
+    </row>
+    <row r="473" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A473" t="s">
+        <v>1309</v>
+      </c>
+      <c r="B473" t="s">
+        <v>1310</v>
+      </c>
+      <c r="C473" t="s">
+        <v>1311</v>
+      </c>
+    </row>
+    <row r="474" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A474" t="s">
+        <v>1312</v>
+      </c>
+      <c r="B474" t="s">
+        <v>1161</v>
+      </c>
+      <c r="C474" t="s">
+        <v>1162</v>
+      </c>
+    </row>
+    <row r="475" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A475" t="s">
+        <v>1313</v>
+      </c>
+      <c r="B475" t="s">
+        <v>1314</v>
+      </c>
+      <c r="C475" t="s">
+        <v>1315</v>
+      </c>
+    </row>
+    <row r="476" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A476" t="s">
+        <v>1316</v>
+      </c>
+      <c r="B476" t="s">
+        <v>1317</v>
+      </c>
+      <c r="C476" t="s">
+        <v>1318</v>
+      </c>
+    </row>
+    <row r="477" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A477" t="s">
+        <v>1319</v>
+      </c>
+      <c r="B477" t="s">
+        <v>1320</v>
+      </c>
+      <c r="C477" t="s">
+        <v>1321</v>
+      </c>
+    </row>
+    <row r="478" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A478" t="s">
+        <v>1322</v>
+      </c>
+      <c r="B478" t="s">
+        <v>1323</v>
+      </c>
+      <c r="C478" t="s">
+        <v>1324</v>
+      </c>
+    </row>
+    <row r="479" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A479" t="s">
+        <v>1325</v>
+      </c>
+      <c r="B479" t="s">
+        <v>1326</v>
+      </c>
+      <c r="C479" t="s">
+        <v>1327</v>
+      </c>
+    </row>
+    <row r="480" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A480" t="s">
+        <v>1328</v>
+      </c>
+      <c r="B480" t="s">
+        <v>1329</v>
+      </c>
+      <c r="C480" t="s">
+        <v>1330</v>
+      </c>
+    </row>
+    <row r="481" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A481" t="s">
+        <v>1331</v>
+      </c>
+      <c r="B481" t="s">
+        <v>1332</v>
+      </c>
+      <c r="C481" t="s">
+        <v>1333</v>
+      </c>
+    </row>
+    <row r="482" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A482" t="s">
+        <v>1334</v>
+      </c>
+      <c r="B482" t="s">
+        <v>1335</v>
+      </c>
+      <c r="C482" t="s">
+        <v>1336</v>
+      </c>
+    </row>
+    <row r="483" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A483" t="s">
+        <v>1337</v>
+      </c>
+      <c r="B483" t="s">
+        <v>1338</v>
+      </c>
+      <c r="C483" t="s">
+        <v>1339</v>
+      </c>
+    </row>
+    <row r="484" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A484" t="s">
+        <v>1340</v>
+      </c>
+      <c r="B484" t="s">
+        <v>1341</v>
+      </c>
+      <c r="C484" t="s">
+        <v>1342</v>
+      </c>
+    </row>
+    <row r="485" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A485" t="s">
+        <v>1343</v>
+      </c>
+      <c r="B485" t="s">
+        <v>1344</v>
+      </c>
+      <c r="C485" t="s">
+        <v>1345</v>
+      </c>
+    </row>
+    <row r="486" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A486" t="s">
+        <v>1346</v>
+      </c>
+      <c r="B486" t="s">
+        <v>1347</v>
+      </c>
+      <c r="C486" t="s">
+        <v>1348</v>
+      </c>
+    </row>
+    <row r="487" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A487" t="s">
+        <v>1349</v>
+      </c>
+      <c r="B487" t="s">
+        <v>1350</v>
+      </c>
+      <c r="C487" t="s">
+        <v>1351</v>
+      </c>
+    </row>
+    <row r="488" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A488" t="s">
+        <v>1352</v>
+      </c>
+      <c r="B488" t="s">
+        <v>1353</v>
+      </c>
+      <c r="C488" t="s">
+        <v>1354</v>
+      </c>
+    </row>
+    <row r="489" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A489" t="s">
+        <v>1355</v>
+      </c>
+      <c r="B489" t="s">
+        <v>1356</v>
+      </c>
+      <c r="C489" t="s">
+        <v>1357</v>
+      </c>
+    </row>
+    <row r="490" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A490" t="s">
+        <v>1358</v>
+      </c>
+      <c r="B490" t="s">
+        <v>1359</v>
+      </c>
+      <c r="C490" t="s">
+        <v>1360</v>
+      </c>
+    </row>
+    <row r="491" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A491" t="s">
+        <v>1361</v>
+      </c>
+      <c r="B491" t="s">
+        <v>1362</v>
+      </c>
+      <c r="C491" t="s">
+        <v>1363</v>
+      </c>
+    </row>
+    <row r="492" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A492" t="s">
+        <v>1364</v>
+      </c>
+      <c r="B492" t="s">
+        <v>1365</v>
+      </c>
+      <c r="C492" t="s">
+        <v>1366</v>
+      </c>
+    </row>
+    <row r="493" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A493" t="s">
+        <v>1367</v>
+      </c>
+      <c r="B493" t="s">
+        <v>1368</v>
+      </c>
+      <c r="C493" t="s">
+        <v>1369</v>
+      </c>
+    </row>
+    <row r="494" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A494" t="s">
+        <v>1370</v>
+      </c>
+      <c r="B494" t="s">
+        <v>1371</v>
+      </c>
+      <c r="C494" t="s">
+        <v>1372</v>
+      </c>
+    </row>
+    <row r="495" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A495" t="s">
+        <v>1373</v>
+      </c>
+      <c r="B495" t="s">
+        <v>1374</v>
+      </c>
+      <c r="C495" t="s">
+        <v>1375</v>
+      </c>
+    </row>
+    <row r="496" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A496" t="s">
+        <v>1376</v>
+      </c>
+      <c r="B496" t="s">
+        <v>1377</v>
+      </c>
+      <c r="C496" t="s">
+        <v>1378</v>
+      </c>
+    </row>
+    <row r="497" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A497" t="s">
+        <v>1379</v>
+      </c>
+      <c r="B497" t="s">
+        <v>1380</v>
+      </c>
+      <c r="C497" t="s">
+        <v>1381</v>
+      </c>
+    </row>
+    <row r="498" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A498" t="s">
+        <v>1382</v>
+      </c>
+      <c r="B498" t="s">
+        <v>1383</v>
+      </c>
+      <c r="C498" t="s">
+        <v>1384</v>
+      </c>
+    </row>
+    <row r="499" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A499" t="s">
+        <v>1385</v>
+      </c>
+      <c r="B499" t="s">
+        <v>1386</v>
+      </c>
+      <c r="C499" t="s">
+        <v>1387</v>
+      </c>
+    </row>
+    <row r="500" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A500" t="s">
+        <v>1388</v>
+      </c>
+      <c r="B500" t="s">
+        <v>1389</v>
+      </c>
+      <c r="C500" t="s">
+        <v>1390</v>
+      </c>
+    </row>
+    <row r="501" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A501" t="s">
+        <v>1391</v>
+      </c>
+      <c r="B501" t="s">
+        <v>1392</v>
+      </c>
+      <c r="C501" t="s">
+        <v>1393</v>
+      </c>
+    </row>
+    <row r="502" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A502" t="s">
+        <v>1394</v>
+      </c>
+      <c r="B502" t="s">
+        <v>1395</v>
+      </c>
+      <c r="C502" t="s">
+        <v>1396</v>
+      </c>
+    </row>
+    <row r="503" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A503" t="s">
+        <v>1397</v>
+      </c>
+      <c r="B503" t="s">
+        <v>1398</v>
+      </c>
+      <c r="C503" t="s">
+        <v>1399</v>
+      </c>
+    </row>
+    <row r="504" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A504" t="s">
+        <v>1400</v>
+      </c>
+      <c r="B504" t="s">
+        <v>1401</v>
+      </c>
+      <c r="C504" t="s">
+        <v>1402</v>
+      </c>
+    </row>
+    <row r="505" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A505" t="s">
+        <v>1403</v>
+      </c>
+      <c r="B505" t="s">
+        <v>1404</v>
+      </c>
+      <c r="C505" t="s">
+        <v>1405</v>
+      </c>
+    </row>
+    <row r="506" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A506" t="s">
+        <v>1406</v>
+      </c>
+      <c r="B506" t="s">
+        <v>1407</v>
+      </c>
+      <c r="C506" t="s">
+        <v>1408</v>
+      </c>
+    </row>
+    <row r="507" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A507" t="s">
+        <v>1409</v>
+      </c>
+      <c r="B507" t="s">
+        <v>1410</v>
+      </c>
+      <c r="C507" t="s">
+        <v>1411</v>
+      </c>
+    </row>
+    <row r="508" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A508" t="s">
+        <v>1412</v>
+      </c>
+      <c r="B508" t="s">
+        <v>1413</v>
+      </c>
+      <c r="C508" t="s">
+        <v>1414</v>
+      </c>
+    </row>
+    <row r="509" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A509" t="s">
+        <v>1415</v>
+      </c>
+      <c r="B509" t="s">
+        <v>1416</v>
+      </c>
+      <c r="C509" t="s">
+        <v>1417</v>
+      </c>
+    </row>
+    <row r="510" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A510" t="s">
+        <v>1418</v>
+      </c>
+      <c r="B510" t="s">
+        <v>1419</v>
+      </c>
+      <c r="C510" t="s">
+        <v>1420</v>
+      </c>
+    </row>
+    <row r="511" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A511" t="s">
+        <v>1421</v>
+      </c>
+      <c r="B511" t="s">
+        <v>1422</v>
+      </c>
+      <c r="C511" t="s">
+        <v>1423</v>
+      </c>
+    </row>
+    <row r="512" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A512" t="s">
+        <v>1424</v>
+      </c>
+      <c r="B512" t="s">
+        <v>1425</v>
+      </c>
+      <c r="C512" t="s">
+        <v>1426</v>
+      </c>
+    </row>
+    <row r="513" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A513" t="s">
+        <v>1427</v>
+      </c>
+      <c r="B513" t="s">
+        <v>1428</v>
+      </c>
+      <c r="C513" t="s">
+        <v>1429</v>
+      </c>
+    </row>
+    <row r="514" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A514" t="s">
+        <v>1430</v>
+      </c>
+      <c r="B514" t="s">
+        <v>1431</v>
+      </c>
+      <c r="C514" t="s">
+        <v>1432</v>
+      </c>
+    </row>
+    <row r="515" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A515" t="s">
+        <v>1433</v>
+      </c>
+      <c r="B515" t="s">
+        <v>1434</v>
+      </c>
+      <c r="C515" t="s">
+        <v>1435</v>
+      </c>
+    </row>
+    <row r="516" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A516" t="s">
+        <v>1436</v>
+      </c>
+      <c r="B516" t="s">
+        <v>1437</v>
+      </c>
+      <c r="C516" t="s">
+        <v>1438</v>
+      </c>
+    </row>
+    <row r="517" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A517" t="s">
+        <v>1439</v>
+      </c>
+      <c r="B517" t="s">
+        <v>1440</v>
+      </c>
+      <c r="C517" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="518" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A518" t="s">
+        <v>1442</v>
+      </c>
+      <c r="B518" t="s">
+        <v>1416</v>
+      </c>
+      <c r="C518" t="s">
+        <v>1417</v>
+      </c>
+    </row>
+    <row r="519" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A519" t="s">
+        <v>1443</v>
+      </c>
+      <c r="B519" t="s">
+        <v>1444</v>
+      </c>
+      <c r="C519" t="s">
+        <v>1445</v>
+      </c>
+    </row>
+    <row r="520" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A520" t="s">
+        <v>1446</v>
+      </c>
+      <c r="B520" t="s">
+        <v>1447</v>
+      </c>
+      <c r="C520" t="s">
+        <v>1448</v>
+      </c>
+    </row>
+    <row r="521" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A521" t="s">
+        <v>1449</v>
+      </c>
+      <c r="B521" t="s">
+        <v>1450</v>
+      </c>
+      <c r="C521" t="s">
+        <v>1451</v>
+      </c>
+    </row>
+    <row r="522" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A522" t="s">
+        <v>1452</v>
+      </c>
+      <c r="B522" t="s">
+        <v>1453</v>
+      </c>
+      <c r="C522" t="s">
+        <v>1454</v>
+      </c>
+    </row>
+    <row r="523" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A523" t="s">
+        <v>1455</v>
+      </c>
+      <c r="B523" t="s">
+        <v>1456</v>
+      </c>
+      <c r="C523" t="s">
+        <v>1457</v>
+      </c>
+    </row>
+    <row r="524" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A524" t="s">
+        <v>1458</v>
+      </c>
+      <c r="B524" t="s">
+        <v>1459</v>
+      </c>
+      <c r="C524" t="s">
+        <v>1460</v>
+      </c>
+    </row>
+    <row r="525" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A525" t="s">
+        <v>1461</v>
+      </c>
+      <c r="B525" t="s">
+        <v>1462</v>
+      </c>
+      <c r="C525" t="s">
+        <v>1463</v>
+      </c>
+    </row>
+    <row r="526" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A526" t="s">
+        <v>1464</v>
+      </c>
+      <c r="B526" t="s">
+        <v>1465</v>
+      </c>
+      <c r="C526" t="s">
+        <v>1466</v>
+      </c>
+    </row>
+    <row r="527" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A527" t="s">
+        <v>1467</v>
+      </c>
+      <c r="B527" t="s">
+        <v>1468</v>
+      </c>
+      <c r="C527" t="s">
+        <v>1469</v>
+      </c>
+    </row>
+    <row r="528" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A528" t="s">
+        <v>1470</v>
+      </c>
+      <c r="B528" t="s">
+        <v>1471</v>
+      </c>
+      <c r="C528" t="s">
+        <v>1472</v>
+      </c>
+    </row>
+    <row r="529" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A529" t="s">
+        <v>1473</v>
+      </c>
+      <c r="B529" t="s">
+        <v>1474</v>
+      </c>
+      <c r="C529" t="s">
+        <v>1475</v>
+      </c>
+    </row>
+    <row r="530" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A530" t="s">
+        <v>1476</v>
+      </c>
+      <c r="B530" t="s">
+        <v>1477</v>
+      </c>
+      <c r="C530" t="s">
+        <v>1478</v>
+      </c>
+    </row>
+    <row r="531" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A531" t="s">
+        <v>1479</v>
+      </c>
+      <c r="B531" t="s">
+        <v>1480</v>
+      </c>
+      <c r="C531" t="s">
+        <v>1481</v>
+      </c>
+    </row>
+    <row r="532" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A532" t="s">
+        <v>1482</v>
+      </c>
+      <c r="B532" t="s">
+        <v>1483</v>
+      </c>
+      <c r="C532" t="s">
+        <v>1484</v>
+      </c>
+    </row>
+    <row r="533" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A533" t="s">
+        <v>1485</v>
+      </c>
+      <c r="B533" t="s">
+        <v>223</v>
+      </c>
+      <c r="C533" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="534" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A534" t="s">
+        <v>1486</v>
+      </c>
+      <c r="B534" t="s">
+        <v>1487</v>
+      </c>
+      <c r="C534" t="s">
+        <v>1488</v>
+      </c>
+    </row>
+    <row r="535" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A535" t="s">
+        <v>1489</v>
+      </c>
+      <c r="B535" t="s">
+        <v>1490</v>
+      </c>
+      <c r="C535" t="s">
+        <v>1491</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>

</xml_diff>

<commit_message>
fix(i18n): seed carries the self-attestation wording for the licence step (en, ru)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/api/prisma/seed/translations_seed.xlsx
+++ b/apps/api/prisma/seed/translations_seed.xlsx
@@ -2032,19 +2032,19 @@
     <t>onboarding.verification.item.license</t>
   </si>
   <si>
-    <t>License &amp; identity verification</t>
-  </si>
-  <si>
-    <t>Верификация лицензии и личности</t>
+    <t>License confirmation</t>
+  </si>
+  <si>
+    <t>Подтверждение лицензии</t>
   </si>
   <si>
     <t>onboarding.verification.item.license.desc</t>
   </si>
   <si>
-    <t>Bar license number and a quick identity check.</t>
-  </si>
-  <si>
-    <t>Номер лицензии адвоката и быстрая проверка личности.</t>
+    <t>Your state and bar number, confirmed with one tick.</t>
+  </si>
+  <si>
+    <t>Штат и номер лицензии — подтверждаете одной галочкой.</t>
   </si>
   <si>
     <t>onboarding.verification.item.subscription</t>

</xml_diff>

<commit_message>
feat(admin): Деньги → Планы page; plan toggles reach subscribers at once
The owner assembles each plan from the entitlement catalog, prices it,
archives it and pushes terms. Switching an entitlement on or off now
applies to everyone on the plan immediately (applyNow, default true);
prices still move only through "apply to subscribers". Adds the
platform_payments entitlement and the friendly texts for plan errors.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013HzzZgU2aHRfxUdBN84yAB
</commit_message>
<xml_diff>
--- a/apps/api/prisma/seed/translations_seed.xlsx
+++ b/apps/api/prisma/seed/translations_seed.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2070" uniqueCount="1909">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2214" uniqueCount="2050">
   <si>
     <t>key</t>
   </si>
@@ -5738,6 +5738,429 @@
   </si>
   <si>
     <t>Выбрать практики</t>
+  </si>
+  <si>
+    <t>plan.free</t>
+  </si>
+  <si>
+    <t>Free</t>
+  </si>
+  <si>
+    <t>Бесплатно</t>
+  </si>
+  <si>
+    <t>plan.status.yours</t>
+  </si>
+  <si>
+    <t>Your plan</t>
+  </si>
+  <si>
+    <t>Ваш план</t>
+  </si>
+  <si>
+    <t>plan.pay.trialDays</t>
+  </si>
+  <si>
+    <t>Start {n} days free</t>
+  </si>
+  <si>
+    <t>Начать {n} дней бесплатно</t>
+  </si>
+  <si>
+    <t>plan.f.seatsIncluded</t>
+  </si>
+  <si>
+    <t>Assistants included: {n}</t>
+  </si>
+  <si>
+    <t>Помощников включено: {n}</t>
+  </si>
+  <si>
+    <t>plan.f.extraSeat</t>
+  </si>
+  <si>
+    <t>Extra assistant: {price}/mo</t>
+  </si>
+  <si>
+    <t>Доп. помощник: {price}/мес</t>
+  </si>
+  <si>
+    <t>plan.f.bidsAnyState</t>
+  </si>
+  <si>
+    <t>Offers in any state</t>
+  </si>
+  <si>
+    <t>Ставки в любом штате</t>
+  </si>
+  <si>
+    <t>plan.f.maxActiveBids</t>
+  </si>
+  <si>
+    <t>Active offers: up to {n}</t>
+  </si>
+  <si>
+    <t>Активных ставок: до {n}</t>
+  </si>
+  <si>
+    <t>plan.f.unlimitedBids</t>
+  </si>
+  <si>
+    <t>Unlimited active offers</t>
+  </si>
+  <si>
+    <t>Активные ставки без ограничений</t>
+  </si>
+  <si>
+    <t>plan.f.prioritySearch</t>
+  </si>
+  <si>
+    <t>Higher in search</t>
+  </si>
+  <si>
+    <t>Приоритет в поиске</t>
+  </si>
+  <si>
+    <t>plan.f.videoCalls</t>
+  </si>
+  <si>
+    <t>Video calls</t>
+  </si>
+  <si>
+    <t>Видеозвонки</t>
+  </si>
+  <si>
+    <t>plan.f.documentTemplates</t>
+  </si>
+  <si>
+    <t>Document templates</t>
+  </si>
+  <si>
+    <t>Шаблоны документов</t>
+  </si>
+  <si>
+    <t>plan.f.trial</t>
+  </si>
+  <si>
+    <t>{n}-day free trial</t>
+  </si>
+  <si>
+    <t>Пробный период {n} дней</t>
+  </si>
+  <si>
+    <t>plan.f.verifiedBadge</t>
+  </si>
+  <si>
+    <t>Verified badge included</t>
+  </si>
+  <si>
+    <t>Галочка верификации включена</t>
+  </si>
+  <si>
+    <t>plan.f.priorityFeed</t>
+  </si>
+  <si>
+    <t>Your cases shown first to attorneys</t>
+  </si>
+  <si>
+    <t>Ваши кейсы — первыми в ленте адвокатов</t>
+  </si>
+  <si>
+    <t>plan.f.maxActiveCases</t>
+  </si>
+  <si>
+    <t>Open cases: up to {n}</t>
+  </si>
+  <si>
+    <t>Открытых кейсов: до {n}</t>
+  </si>
+  <si>
+    <t>plan.f.unlimitedCases</t>
+  </si>
+  <si>
+    <t>Unlimited open cases</t>
+  </si>
+  <si>
+    <t>Открытые кейсы без ограничений</t>
+  </si>
+  <si>
+    <t>plan.seats.extra</t>
+  </si>
+  <si>
+    <t>Extra assistants</t>
+  </si>
+  <si>
+    <t>Доп. помощники</t>
+  </si>
+  <si>
+    <t>plan.seats.each</t>
+  </si>
+  <si>
+    <t>+{price} a month each</t>
+  </si>
+  <si>
+    <t>+{price} в месяц за каждого</t>
+  </si>
+  <si>
+    <t>plan.seats.includedN</t>
+  </si>
+  <si>
+    <t>Included in the plan: {n}</t>
+  </si>
+  <si>
+    <t>Включено в план: {n}</t>
+  </si>
+  <si>
+    <t>plan.seats.limit</t>
+  </si>
+  <si>
+    <t>You can add {n} more</t>
+  </si>
+  <si>
+    <t>Можно добавить ещё: {n}</t>
+  </si>
+  <si>
+    <t>plan.current.title</t>
+  </si>
+  <si>
+    <t>plan.current.includes</t>
+  </si>
+  <si>
+    <t>What's included</t>
+  </si>
+  <si>
+    <t>Что входит</t>
+  </si>
+  <si>
+    <t>plan.seats.summary</t>
+  </si>
+  <si>
+    <t>Assistants: {total} · {included} included, {extra} extra</t>
+  </si>
+  <si>
+    <t>Помощники: {total} · включено {included}, доп. {extra}</t>
+  </si>
+  <si>
+    <t>plan.seats.summary.max</t>
+  </si>
+  <si>
+    <t>Seat limit: {max}</t>
+  </si>
+  <si>
+    <t>Максимум мест: {max}</t>
+  </si>
+  <si>
+    <t>plan.client.title</t>
+  </si>
+  <si>
+    <t>Client subscription</t>
+  </si>
+  <si>
+    <t>Подписка клиента</t>
+  </si>
+  <si>
+    <t>plan.client.hint</t>
+  </si>
+  <si>
+    <t>Badge, priority in the feed, case limits</t>
+  </si>
+  <si>
+    <t>Галочка, приоритет в ленте, лимиты кейсов</t>
+  </si>
+  <si>
+    <t>plan.client.choose</t>
+  </si>
+  <si>
+    <t>Choose a plan</t>
+  </si>
+  <si>
+    <t>Выберите план</t>
+  </si>
+  <si>
+    <t>plan.client.subscribe</t>
+  </si>
+  <si>
+    <t>Subscribe</t>
+  </si>
+  <si>
+    <t>Оформить</t>
+  </si>
+  <si>
+    <t>plan.client.subscribeTrial</t>
+  </si>
+  <si>
+    <t>Subscribe · {n} days free</t>
+  </si>
+  <si>
+    <t>Оформить · {n} дней бесплатно</t>
+  </si>
+  <si>
+    <t>plan.client.cancel</t>
+  </si>
+  <si>
+    <t>Отменить</t>
+  </si>
+  <si>
+    <t>plan.client.resume</t>
+  </si>
+  <si>
+    <t>Resume</t>
+  </si>
+  <si>
+    <t>Возобновить</t>
+  </si>
+  <si>
+    <t>plan.client.trialHint</t>
+  </si>
+  <si>
+    <t>Your first purchase of a plan with a trial is free for the trial days.</t>
+  </si>
+  <si>
+    <t>Первая покупка плана с пробным периодом — бесплатно на время триала.</t>
+  </si>
+  <si>
+    <t>plan.client.line.trialEnds</t>
+  </si>
+  <si>
+    <t>Trial until {date}, then {price}</t>
+  </si>
+  <si>
+    <t>Пробный период до {date}, затем {price}</t>
+  </si>
+  <si>
+    <t>plan.client.line.nextCharge</t>
+  </si>
+  <si>
+    <t>Next charge {date} — {price}</t>
+  </si>
+  <si>
+    <t>Следующее списание {date} — {price}</t>
+  </si>
+  <si>
+    <t>plan.client.line.cancelScheduled</t>
+  </si>
+  <si>
+    <t>Ends on {date}</t>
+  </si>
+  <si>
+    <t>Подписка закончится {date}</t>
+  </si>
+  <si>
+    <t>plan.client.line.pastDue</t>
+  </si>
+  <si>
+    <t>Payment failed — update your card</t>
+  </si>
+  <si>
+    <t>Оплата не прошла — обновите карту</t>
+  </si>
+  <si>
+    <t>plan.client.line.ended</t>
+  </si>
+  <si>
+    <t>Subscription ended</t>
+  </si>
+  <si>
+    <t>Подписка завершена</t>
+  </si>
+  <si>
+    <t>plan.client.cancel.title</t>
+  </si>
+  <si>
+    <t>Cancel the subscription?</t>
+  </si>
+  <si>
+    <t>Отменить подписку?</t>
+  </si>
+  <si>
+    <t>plan.client.cancel.body</t>
+  </si>
+  <si>
+    <t>Access stays until {date}.</t>
+  </si>
+  <si>
+    <t>Доступ сохранится до {date}.</t>
+  </si>
+  <si>
+    <t>plan.client.cancel.bodyNoDate</t>
+  </si>
+  <si>
+    <t>Access stays until the end of the paid period.</t>
+  </si>
+  <si>
+    <t>Доступ сохранится до конца оплаченного периода.</t>
+  </si>
+  <si>
+    <t>plan.client.cancel.done</t>
+  </si>
+  <si>
+    <t>Won't renew</t>
+  </si>
+  <si>
+    <t>Подписка не продлится</t>
+  </si>
+  <si>
+    <t>plan.client.resume.done</t>
+  </si>
+  <si>
+    <t>Subscription resumed</t>
+  </si>
+  <si>
+    <t>Подписка возобновлена</t>
+  </si>
+  <si>
+    <t>plan.client.done.active</t>
+  </si>
+  <si>
+    <t>Subscription active</t>
+  </si>
+  <si>
+    <t>Подписка оформлена</t>
+  </si>
+  <si>
+    <t>plan.client.done.trial</t>
+  </si>
+  <si>
+    <t>Your trial has started</t>
+  </si>
+  <si>
+    <t>Пробный период начался</t>
+  </si>
+  <si>
+    <t>plan.client.noPlans</t>
+  </si>
+  <si>
+    <t>No client plans yet</t>
+  </si>
+  <si>
+    <t>Пока нет планов для клиентов</t>
+  </si>
+  <si>
+    <t>plan.badge.included</t>
+  </si>
+  <si>
+    <t>The badge is included in your plan</t>
+  </si>
+  <si>
+    <t>Галочка включена в ваш план</t>
+  </si>
+  <si>
+    <t>plan.badge.included.hint</t>
+  </si>
+  <si>
+    <t>Once your documents are approved the badge shows — no separate payment.</t>
+  </si>
+  <si>
+    <t>После проверки документов галочка появится без отдельной оплаты.</t>
+  </si>
+  <si>
+    <t>plan.feed.priority</t>
+  </si>
+  <si>
+    <t>PRIORITY</t>
+  </si>
+  <si>
+    <t>ПРИОРИТЕТ</t>
   </si>
 </sst>
 </file>
@@ -6114,7 +6537,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C690"/>
+  <dimension ref="A1:C738"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -13711,6 +14134,534 @@
         <v>1908</v>
       </c>
     </row>
+    <row r="691" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A691" t="s">
+        <v>1909</v>
+      </c>
+      <c r="B691" t="s">
+        <v>1910</v>
+      </c>
+      <c r="C691" t="s">
+        <v>1911</v>
+      </c>
+    </row>
+    <row r="692" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A692" t="s">
+        <v>1912</v>
+      </c>
+      <c r="B692" t="s">
+        <v>1913</v>
+      </c>
+      <c r="C692" t="s">
+        <v>1914</v>
+      </c>
+    </row>
+    <row r="693" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A693" t="s">
+        <v>1915</v>
+      </c>
+      <c r="B693" t="s">
+        <v>1916</v>
+      </c>
+      <c r="C693" t="s">
+        <v>1917</v>
+      </c>
+    </row>
+    <row r="694" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A694" t="s">
+        <v>1918</v>
+      </c>
+      <c r="B694" t="s">
+        <v>1919</v>
+      </c>
+      <c r="C694" t="s">
+        <v>1920</v>
+      </c>
+    </row>
+    <row r="695" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A695" t="s">
+        <v>1921</v>
+      </c>
+      <c r="B695" t="s">
+        <v>1922</v>
+      </c>
+      <c r="C695" t="s">
+        <v>1923</v>
+      </c>
+    </row>
+    <row r="696" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A696" t="s">
+        <v>1924</v>
+      </c>
+      <c r="B696" t="s">
+        <v>1925</v>
+      </c>
+      <c r="C696" t="s">
+        <v>1926</v>
+      </c>
+    </row>
+    <row r="697" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A697" t="s">
+        <v>1927</v>
+      </c>
+      <c r="B697" t="s">
+        <v>1928</v>
+      </c>
+      <c r="C697" t="s">
+        <v>1929</v>
+      </c>
+    </row>
+    <row r="698" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A698" t="s">
+        <v>1930</v>
+      </c>
+      <c r="B698" t="s">
+        <v>1931</v>
+      </c>
+      <c r="C698" t="s">
+        <v>1932</v>
+      </c>
+    </row>
+    <row r="699" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A699" t="s">
+        <v>1933</v>
+      </c>
+      <c r="B699" t="s">
+        <v>1934</v>
+      </c>
+      <c r="C699" t="s">
+        <v>1935</v>
+      </c>
+    </row>
+    <row r="700" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A700" t="s">
+        <v>1936</v>
+      </c>
+      <c r="B700" t="s">
+        <v>1937</v>
+      </c>
+      <c r="C700" t="s">
+        <v>1938</v>
+      </c>
+    </row>
+    <row r="701" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A701" t="s">
+        <v>1939</v>
+      </c>
+      <c r="B701" t="s">
+        <v>1940</v>
+      </c>
+      <c r="C701" t="s">
+        <v>1941</v>
+      </c>
+    </row>
+    <row r="702" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A702" t="s">
+        <v>1942</v>
+      </c>
+      <c r="B702" t="s">
+        <v>1943</v>
+      </c>
+      <c r="C702" t="s">
+        <v>1944</v>
+      </c>
+    </row>
+    <row r="703" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A703" t="s">
+        <v>1945</v>
+      </c>
+      <c r="B703" t="s">
+        <v>1946</v>
+      </c>
+      <c r="C703" t="s">
+        <v>1947</v>
+      </c>
+    </row>
+    <row r="704" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A704" t="s">
+        <v>1948</v>
+      </c>
+      <c r="B704" t="s">
+        <v>1949</v>
+      </c>
+      <c r="C704" t="s">
+        <v>1950</v>
+      </c>
+    </row>
+    <row r="705" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A705" t="s">
+        <v>1951</v>
+      </c>
+      <c r="B705" t="s">
+        <v>1952</v>
+      </c>
+      <c r="C705" t="s">
+        <v>1953</v>
+      </c>
+    </row>
+    <row r="706" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A706" t="s">
+        <v>1954</v>
+      </c>
+      <c r="B706" t="s">
+        <v>1955</v>
+      </c>
+      <c r="C706" t="s">
+        <v>1956</v>
+      </c>
+    </row>
+    <row r="707" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A707" t="s">
+        <v>1957</v>
+      </c>
+      <c r="B707" t="s">
+        <v>1958</v>
+      </c>
+      <c r="C707" t="s">
+        <v>1959</v>
+      </c>
+    </row>
+    <row r="708" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A708" t="s">
+        <v>1960</v>
+      </c>
+      <c r="B708" t="s">
+        <v>1961</v>
+      </c>
+      <c r="C708" t="s">
+        <v>1962</v>
+      </c>
+    </row>
+    <row r="709" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A709" t="s">
+        <v>1963</v>
+      </c>
+      <c r="B709" t="s">
+        <v>1964</v>
+      </c>
+      <c r="C709" t="s">
+        <v>1965</v>
+      </c>
+    </row>
+    <row r="710" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A710" t="s">
+        <v>1966</v>
+      </c>
+      <c r="B710" t="s">
+        <v>1967</v>
+      </c>
+      <c r="C710" t="s">
+        <v>1968</v>
+      </c>
+    </row>
+    <row r="711" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A711" t="s">
+        <v>1969</v>
+      </c>
+      <c r="B711" t="s">
+        <v>1913</v>
+      </c>
+      <c r="C711" t="s">
+        <v>1914</v>
+      </c>
+    </row>
+    <row r="712" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A712" t="s">
+        <v>1970</v>
+      </c>
+      <c r="B712" t="s">
+        <v>1971</v>
+      </c>
+      <c r="C712" t="s">
+        <v>1972</v>
+      </c>
+    </row>
+    <row r="713" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A713" t="s">
+        <v>1973</v>
+      </c>
+      <c r="B713" t="s">
+        <v>1974</v>
+      </c>
+      <c r="C713" t="s">
+        <v>1975</v>
+      </c>
+    </row>
+    <row r="714" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A714" t="s">
+        <v>1976</v>
+      </c>
+      <c r="B714" t="s">
+        <v>1977</v>
+      </c>
+      <c r="C714" t="s">
+        <v>1978</v>
+      </c>
+    </row>
+    <row r="715" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A715" t="s">
+        <v>1979</v>
+      </c>
+      <c r="B715" t="s">
+        <v>1980</v>
+      </c>
+      <c r="C715" t="s">
+        <v>1981</v>
+      </c>
+    </row>
+    <row r="716" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A716" t="s">
+        <v>1982</v>
+      </c>
+      <c r="B716" t="s">
+        <v>1983</v>
+      </c>
+      <c r="C716" t="s">
+        <v>1984</v>
+      </c>
+    </row>
+    <row r="717" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A717" t="s">
+        <v>1985</v>
+      </c>
+      <c r="B717" t="s">
+        <v>1986</v>
+      </c>
+      <c r="C717" t="s">
+        <v>1987</v>
+      </c>
+    </row>
+    <row r="718" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A718" t="s">
+        <v>1988</v>
+      </c>
+      <c r="B718" t="s">
+        <v>1989</v>
+      </c>
+      <c r="C718" t="s">
+        <v>1990</v>
+      </c>
+    </row>
+    <row r="719" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A719" t="s">
+        <v>1991</v>
+      </c>
+      <c r="B719" t="s">
+        <v>1992</v>
+      </c>
+      <c r="C719" t="s">
+        <v>1993</v>
+      </c>
+    </row>
+    <row r="720" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A720" t="s">
+        <v>1994</v>
+      </c>
+      <c r="B720" t="s">
+        <v>95</v>
+      </c>
+      <c r="C720" t="s">
+        <v>1995</v>
+      </c>
+    </row>
+    <row r="721" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A721" t="s">
+        <v>1996</v>
+      </c>
+      <c r="B721" t="s">
+        <v>1997</v>
+      </c>
+      <c r="C721" t="s">
+        <v>1998</v>
+      </c>
+    </row>
+    <row r="722" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A722" t="s">
+        <v>1999</v>
+      </c>
+      <c r="B722" t="s">
+        <v>2000</v>
+      </c>
+      <c r="C722" t="s">
+        <v>2001</v>
+      </c>
+    </row>
+    <row r="723" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A723" t="s">
+        <v>2002</v>
+      </c>
+      <c r="B723" t="s">
+        <v>2003</v>
+      </c>
+      <c r="C723" t="s">
+        <v>2004</v>
+      </c>
+    </row>
+    <row r="724" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A724" t="s">
+        <v>2005</v>
+      </c>
+      <c r="B724" t="s">
+        <v>2006</v>
+      </c>
+      <c r="C724" t="s">
+        <v>2007</v>
+      </c>
+    </row>
+    <row r="725" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A725" t="s">
+        <v>2008</v>
+      </c>
+      <c r="B725" t="s">
+        <v>2009</v>
+      </c>
+      <c r="C725" t="s">
+        <v>2010</v>
+      </c>
+    </row>
+    <row r="726" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A726" t="s">
+        <v>2011</v>
+      </c>
+      <c r="B726" t="s">
+        <v>2012</v>
+      </c>
+      <c r="C726" t="s">
+        <v>2013</v>
+      </c>
+    </row>
+    <row r="727" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A727" t="s">
+        <v>2014</v>
+      </c>
+      <c r="B727" t="s">
+        <v>2015</v>
+      </c>
+      <c r="C727" t="s">
+        <v>2016</v>
+      </c>
+    </row>
+    <row r="728" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A728" t="s">
+        <v>2017</v>
+      </c>
+      <c r="B728" t="s">
+        <v>2018</v>
+      </c>
+      <c r="C728" t="s">
+        <v>2019</v>
+      </c>
+    </row>
+    <row r="729" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A729" t="s">
+        <v>2020</v>
+      </c>
+      <c r="B729" t="s">
+        <v>2021</v>
+      </c>
+      <c r="C729" t="s">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="730" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A730" t="s">
+        <v>2023</v>
+      </c>
+      <c r="B730" t="s">
+        <v>2024</v>
+      </c>
+      <c r="C730" t="s">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="731" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A731" t="s">
+        <v>2026</v>
+      </c>
+      <c r="B731" t="s">
+        <v>2027</v>
+      </c>
+      <c r="C731" t="s">
+        <v>2028</v>
+      </c>
+    </row>
+    <row r="732" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A732" t="s">
+        <v>2029</v>
+      </c>
+      <c r="B732" t="s">
+        <v>2030</v>
+      </c>
+      <c r="C732" t="s">
+        <v>2031</v>
+      </c>
+    </row>
+    <row r="733" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A733" t="s">
+        <v>2032</v>
+      </c>
+      <c r="B733" t="s">
+        <v>2033</v>
+      </c>
+      <c r="C733" t="s">
+        <v>2034</v>
+      </c>
+    </row>
+    <row r="734" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A734" t="s">
+        <v>2035</v>
+      </c>
+      <c r="B734" t="s">
+        <v>2036</v>
+      </c>
+      <c r="C734" t="s">
+        <v>2037</v>
+      </c>
+    </row>
+    <row r="735" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A735" t="s">
+        <v>2038</v>
+      </c>
+      <c r="B735" t="s">
+        <v>2039</v>
+      </c>
+      <c r="C735" t="s">
+        <v>2040</v>
+      </c>
+    </row>
+    <row r="736" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A736" t="s">
+        <v>2041</v>
+      </c>
+      <c r="B736" t="s">
+        <v>2042</v>
+      </c>
+      <c r="C736" t="s">
+        <v>2043</v>
+      </c>
+    </row>
+    <row r="737" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A737" t="s">
+        <v>2044</v>
+      </c>
+      <c r="B737" t="s">
+        <v>2045</v>
+      </c>
+      <c r="C737" t="s">
+        <v>2046</v>
+      </c>
+    </row>
+    <row r="738" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A738" t="s">
+        <v>2047</v>
+      </c>
+      <c r="B738" t="s">
+        <v>2048</v>
+      </c>
+      <c r="C738" t="s">
+        <v>2049</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>

</xml_diff>

<commit_message>
fix(mobile): new plan error codes in the app list, with en + ru texts
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013HzzZgU2aHRfxUdBN84yAB
</commit_message>
<xml_diff>
--- a/apps/api/prisma/seed/translations_seed.xlsx
+++ b/apps/api/prisma/seed/translations_seed.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2238" uniqueCount="2074">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2250" uniqueCount="2086">
   <si>
     <t>key</t>
   </si>
@@ -6233,6 +6233,42 @@
   </si>
   <si>
     <t>Продвижение кейсов</t>
+  </si>
+  <si>
+    <t>error.api.ENTITLEMENT_REQUIRED</t>
+  </si>
+  <si>
+    <t>This feature is not part of your plan.</t>
+  </si>
+  <si>
+    <t>Эта возможность не входит в ваш план.</t>
+  </si>
+  <si>
+    <t>error.api.BID_LIMIT_REACHED</t>
+  </si>
+  <si>
+    <t>You've reached your plan's limit of active offers.</t>
+  </si>
+  <si>
+    <t>Достигнут лимит активных ставок вашего плана.</t>
+  </si>
+  <si>
+    <t>error.api.CASE_LIMIT_REACHED</t>
+  </si>
+  <si>
+    <t>You've reached your plan's limit of open cases.</t>
+  </si>
+  <si>
+    <t>Достигнут лимит открытых кейсов вашего плана.</t>
+  </si>
+  <si>
+    <t>error.api.PLAN_NOT_AVAILABLE</t>
+  </si>
+  <si>
+    <t>This plan is not available right now. Refresh the screen.</t>
+  </si>
+  <si>
+    <t>Этот план сейчас недоступен. Обновите экран.</t>
   </si>
 </sst>
 </file>
@@ -6609,7 +6645,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C746"/>
+  <dimension ref="A1:C750"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -14822,6 +14858,50 @@
         <v>2073</v>
       </c>
     </row>
+    <row r="747" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A747" t="s">
+        <v>2074</v>
+      </c>
+      <c r="B747" t="s">
+        <v>2075</v>
+      </c>
+      <c r="C747" t="s">
+        <v>2076</v>
+      </c>
+    </row>
+    <row r="748" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A748" t="s">
+        <v>2077</v>
+      </c>
+      <c r="B748" t="s">
+        <v>2078</v>
+      </c>
+      <c r="C748" t="s">
+        <v>2079</v>
+      </c>
+    </row>
+    <row r="749" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A749" t="s">
+        <v>2080</v>
+      </c>
+      <c r="B749" t="s">
+        <v>2081</v>
+      </c>
+      <c r="C749" t="s">
+        <v>2082</v>
+      </c>
+    </row>
+    <row r="750" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A750" t="s">
+        <v>2083</v>
+      </c>
+      <c r="B750" t="s">
+        <v>2084</v>
+      </c>
+      <c r="C750" t="s">
+        <v>2085</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>

</xml_diff>

<commit_message>
i18n: case screens in all languages after an audit — 65 keys that were English outside ru/en, zh-tw gaps, back-translation fixes (ne, ar, he, hi, ko, ja, de, th, ru), RTL arrows and gaps; strings also in the seed file
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/api/prisma/seed/translations_seed.xlsx
+++ b/apps/api/prisma/seed/translations_seed.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2253" uniqueCount="2089">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2712" uniqueCount="2511">
   <si>
     <t>key</t>
   </si>
@@ -6278,6 +6278,1272 @@
   </si>
   <si>
     <t>Этот план сейчас недоступен. Обновите экран.</t>
+  </si>
+  <si>
+    <t>cases.facts.deadline</t>
+  </si>
+  <si>
+    <t>Deadline</t>
+  </si>
+  <si>
+    <t>Срок</t>
+  </si>
+  <si>
+    <t>cases.card.locked</t>
+  </si>
+  <si>
+    <t>locked</t>
+  </si>
+  <si>
+    <t>закрыто</t>
+  </si>
+  <si>
+    <t>cases.card.bid</t>
+  </si>
+  <si>
+    <t>Бид</t>
+  </si>
+  <si>
+    <t>cases.work.chatWithClient</t>
+  </si>
+  <si>
+    <t>Chat with client</t>
+  </si>
+  <si>
+    <t>Чат с клиентом</t>
+  </si>
+  <si>
+    <t>cases.owner.chatWithLawyer</t>
+  </si>
+  <si>
+    <t>Chat with lawyer</t>
+  </si>
+  <si>
+    <t>Чат с юристом</t>
+  </si>
+  <si>
+    <t>cases.status.acceptedByBoth</t>
+  </si>
+  <si>
+    <t>Accepted by both</t>
+  </si>
+  <si>
+    <t>Принят обеими сторонами</t>
+  </si>
+  <si>
+    <t>cases.tab.overview</t>
+  </si>
+  <si>
+    <t>Overview</t>
+  </si>
+  <si>
+    <t>Обзор</t>
+  </si>
+  <si>
+    <t>cases.tab.files</t>
+  </si>
+  <si>
+    <t>Files</t>
+  </si>
+  <si>
+    <t>Файлы</t>
+  </si>
+  <si>
+    <t>cases.tab.tasks</t>
+  </si>
+  <si>
+    <t>Tasks</t>
+  </si>
+  <si>
+    <t>Задачи</t>
+  </si>
+  <si>
+    <t>cases.tab.updates</t>
+  </si>
+  <si>
+    <t>Updates</t>
+  </si>
+  <si>
+    <t>Обновления</t>
+  </si>
+  <si>
+    <t>cases.tab.activity</t>
+  </si>
+  <si>
+    <t>Activity</t>
+  </si>
+  <si>
+    <t>Активность</t>
+  </si>
+  <si>
+    <t>cases.detail.where</t>
+  </si>
+  <si>
+    <t>Where</t>
+  </si>
+  <si>
+    <t>Где</t>
+  </si>
+  <si>
+    <t>cases.files.documents</t>
+  </si>
+  <si>
+    <t>cases.files.photos</t>
+  </si>
+  <si>
+    <t>Photos</t>
+  </si>
+  <si>
+    <t>Фото</t>
+  </si>
+  <si>
+    <t>cases.files.all</t>
+  </si>
+  <si>
+    <t>All</t>
+  </si>
+  <si>
+    <t>Все</t>
+  </si>
+  <si>
+    <t>cases.files.fromTasks</t>
+  </si>
+  <si>
+    <t>From tasks</t>
+  </si>
+  <si>
+    <t>Из задач</t>
+  </si>
+  <si>
+    <t>cases.files.fromUpdates</t>
+  </si>
+  <si>
+    <t>From updates</t>
+  </si>
+  <si>
+    <t>Из обновлений</t>
+  </si>
+  <si>
+    <t>cases.files.samples</t>
+  </si>
+  <si>
+    <t>Samples</t>
+  </si>
+  <si>
+    <t>Образцы</t>
+  </si>
+  <si>
+    <t>cases.files.empty</t>
+  </si>
+  <si>
+    <t>No files yet</t>
+  </si>
+  <si>
+    <t>Файлов пока нет</t>
+  </si>
+  <si>
+    <t>cases.files.photo</t>
+  </si>
+  <si>
+    <t>Photo</t>
+  </si>
+  <si>
+    <t>cases.files.sample</t>
+  </si>
+  <si>
+    <t>Sample</t>
+  </si>
+  <si>
+    <t>Образец</t>
+  </si>
+  <si>
+    <t>cases.files.fromLawyer</t>
+  </si>
+  <si>
+    <t>From lawyer</t>
+  </si>
+  <si>
+    <t>От юриста</t>
+  </si>
+  <si>
+    <t>cases.files.fromTask</t>
+  </si>
+  <si>
+    <t>From task: {title}</t>
+  </si>
+  <si>
+    <t>Из задачи: {title}</t>
+  </si>
+  <si>
+    <t>cases.files.fromUpdate</t>
+  </si>
+  <si>
+    <t>From update</t>
+  </si>
+  <si>
+    <t>Из обновления</t>
+  </si>
+  <si>
+    <t>cases.files.download</t>
+  </si>
+  <si>
+    <t>Download</t>
+  </si>
+  <si>
+    <t>Скачать</t>
+  </si>
+  <si>
+    <t>cases.files.openBtn</t>
+  </si>
+  <si>
+    <t>Open</t>
+  </si>
+  <si>
+    <t>Открыть</t>
+  </si>
+  <si>
+    <t>cases.files.count.one</t>
+  </si>
+  <si>
+    <t>{count} file</t>
+  </si>
+  <si>
+    <t>{count} файл</t>
+  </si>
+  <si>
+    <t>cases.files.count.other</t>
+  </si>
+  <si>
+    <t>{count} files</t>
+  </si>
+  <si>
+    <t>{count} файла</t>
+  </si>
+  <si>
+    <t>cases.role.client</t>
+  </si>
+  <si>
+    <t>cases.role.attorney</t>
+  </si>
+  <si>
+    <t>Licensed Attorney</t>
+  </si>
+  <si>
+    <t>Юрист с лицензией</t>
+  </si>
+  <si>
+    <t>cases.updates.write</t>
+  </si>
+  <si>
+    <t>Write an update…</t>
+  </si>
+  <si>
+    <t>Напишите обновление…</t>
+  </si>
+  <si>
+    <t>cases.updates.me</t>
+  </si>
+  <si>
+    <t>Me</t>
+  </si>
+  <si>
+    <t>Я</t>
+  </si>
+  <si>
+    <t>cases.updates.empty</t>
+  </si>
+  <si>
+    <t>No updates yet</t>
+  </si>
+  <si>
+    <t>Обновлений пока нет</t>
+  </si>
+  <si>
+    <t>cases.updates.taskDone</t>
+  </si>
+  <si>
+    <t>Done: {title}</t>
+  </si>
+  <si>
+    <t>Выполнено: {title}</t>
+  </si>
+  <si>
+    <t>cases.updates.taskFiles</t>
+  </si>
+  <si>
+    <t>Added to the task: {title}</t>
+  </si>
+  <si>
+    <t>Добавлено в задачу: {title}</t>
+  </si>
+  <si>
+    <t>cases.activity.empty</t>
+  </si>
+  <si>
+    <t>Nothing has happened yet</t>
+  </si>
+  <si>
+    <t>Пока ничего не происходило</t>
+  </si>
+  <si>
+    <t>cases.activity.update</t>
+  </si>
+  <si>
+    <t>{name} wrote an update</t>
+  </si>
+  <si>
+    <t>{name} написал(а) обновление</t>
+  </si>
+  <si>
+    <t>cases.activity.taskCreated</t>
+  </si>
+  <si>
+    <t>{name} created the task “{title}”</t>
+  </si>
+  <si>
+    <t>{name} создал(а) задачу «{title}»</t>
+  </si>
+  <si>
+    <t>cases.activity.taskDone</t>
+  </si>
+  <si>
+    <t>{name} completed “{title}”</t>
+  </si>
+  <si>
+    <t>{name} выполнил(а) «{title}»</t>
+  </si>
+  <si>
+    <t>cases.activity.taskUndone</t>
+  </si>
+  <si>
+    <t>{name} unmarked “{title}”</t>
+  </si>
+  <si>
+    <t>{name} снял(а) отметку «{title}»</t>
+  </si>
+  <si>
+    <t>cases.activity.taskClosed</t>
+  </si>
+  <si>
+    <t>{name} closed “{title}”</t>
+  </si>
+  <si>
+    <t>{name} закрыл(а) «{title}»</t>
+  </si>
+  <si>
+    <t>cases.activity.taskReopened</t>
+  </si>
+  <si>
+    <t>{name} reopened “{title}”</t>
+  </si>
+  <si>
+    <t>{name} открыл(а) заново «{title}»</t>
+  </si>
+  <si>
+    <t>cases.activity.filesAdded</t>
+  </si>
+  <si>
+    <t>{name} added {count} files to “{title}”</t>
+  </si>
+  <si>
+    <t>{name} добавил(а) в «{title}» файлы: {count}</t>
+  </si>
+  <si>
+    <t>cases.tasks.forClient</t>
+  </si>
+  <si>
+    <t>For client</t>
+  </si>
+  <si>
+    <t>Для клиента</t>
+  </si>
+  <si>
+    <t>cases.tasks.shared</t>
+  </si>
+  <si>
+    <t>Shared</t>
+  </si>
+  <si>
+    <t>Общие</t>
+  </si>
+  <si>
+    <t>cases.tasks.private</t>
+  </si>
+  <si>
+    <t>Private</t>
+  </si>
+  <si>
+    <t>Личные</t>
+  </si>
+  <si>
+    <t>cases.tasks.yours</t>
+  </si>
+  <si>
+    <t>Your tasks</t>
+  </si>
+  <si>
+    <t>Ваши задачи</t>
+  </si>
+  <si>
+    <t>cases.tasks.lawyerProgress</t>
+  </si>
+  <si>
+    <t>Lawyer's progress</t>
+  </si>
+  <si>
+    <t>Работа юриста</t>
+  </si>
+  <si>
+    <t>cases.tasks.forClientHint</t>
+  </si>
+  <si>
+    <t>The client sees it, answers and attaches files</t>
+  </si>
+  <si>
+    <t>Клиент видит, отвечает и прикладывает файлы</t>
+  </si>
+  <si>
+    <t>cases.tasks.sharedHint</t>
+  </si>
+  <si>
+    <t>The client sees it, only you tick it</t>
+  </si>
+  <si>
+    <t>Клиент видит, отмечаете только вы</t>
+  </si>
+  <si>
+    <t>cases.tasks.privateHint</t>
+  </si>
+  <si>
+    <t>Only for you, the client does not see it</t>
+  </si>
+  <si>
+    <t>Только для вас, клиент не видит</t>
+  </si>
+  <si>
+    <t>cases.tasks.add</t>
+  </si>
+  <si>
+    <t>Task</t>
+  </si>
+  <si>
+    <t>Задача</t>
+  </si>
+  <si>
+    <t>cases.tasks.empty</t>
+  </si>
+  <si>
+    <t>cases.tasks.toDo</t>
+  </si>
+  <si>
+    <t>To do</t>
+  </si>
+  <si>
+    <t>Нужно сделать</t>
+  </si>
+  <si>
+    <t>cases.tasks.waitingClient</t>
+  </si>
+  <si>
+    <t>Waiting for the client</t>
+  </si>
+  <si>
+    <t>Ждём клиента</t>
+  </si>
+  <si>
+    <t>cases.tasks.doneOn</t>
+  </si>
+  <si>
+    <t>Done {date}</t>
+  </si>
+  <si>
+    <t>Выполнено {date}</t>
+  </si>
+  <si>
+    <t>cases.tasks.closedOn</t>
+  </si>
+  <si>
+    <t>Closed {date}</t>
+  </si>
+  <si>
+    <t>Закрыто {date}</t>
+  </si>
+  <si>
+    <t>cases.tasks.progress</t>
+  </si>
+  <si>
+    <t>{done} of {total}</t>
+  </si>
+  <si>
+    <t>{done} из {total}</t>
+  </si>
+  <si>
+    <t>cases.tasks.addFile</t>
+  </si>
+  <si>
+    <t>Add file</t>
+  </si>
+  <si>
+    <t>Добавить файл</t>
+  </si>
+  <si>
+    <t>cases.tasks.addFiles</t>
+  </si>
+  <si>
+    <t>Add files</t>
+  </si>
+  <si>
+    <t>Добавить файлы</t>
+  </si>
+  <si>
+    <t>cases.tasks.addMore</t>
+  </si>
+  <si>
+    <t>Add more</t>
+  </si>
+  <si>
+    <t>Добавить ещё</t>
+  </si>
+  <si>
+    <t>cases.tasks.done</t>
+  </si>
+  <si>
+    <t>cases.tasks.markDone</t>
+  </si>
+  <si>
+    <t>Mark done</t>
+  </si>
+  <si>
+    <t>Отметить выполненной</t>
+  </si>
+  <si>
+    <t>cases.tasks.undo</t>
+  </si>
+  <si>
+    <t>Unmark</t>
+  </si>
+  <si>
+    <t>Снять отметку</t>
+  </si>
+  <si>
+    <t>cases.tasks.close</t>
+  </si>
+  <si>
+    <t>cases.tasks.reopen</t>
+  </si>
+  <si>
+    <t>Reopen</t>
+  </si>
+  <si>
+    <t>Открыть заново</t>
+  </si>
+  <si>
+    <t>cases.compose.newTask</t>
+  </si>
+  <si>
+    <t>New task</t>
+  </si>
+  <si>
+    <t>Новая задача</t>
+  </si>
+  <si>
+    <t>cases.compose.newUpdate</t>
+  </si>
+  <si>
+    <t>New update</t>
+  </si>
+  <si>
+    <t>Новое обновление</t>
+  </si>
+  <si>
+    <t>cases.compose.addFiles</t>
+  </si>
+  <si>
+    <t>cases.compose.create</t>
+  </si>
+  <si>
+    <t>cases.compose.send</t>
+  </si>
+  <si>
+    <t>Send</t>
+  </si>
+  <si>
+    <t>Отправить</t>
+  </si>
+  <si>
+    <t>cases.compose.titleHint</t>
+  </si>
+  <si>
+    <t>Title</t>
+  </si>
+  <si>
+    <t>Название</t>
+  </si>
+  <si>
+    <t>cases.compose.taskHint</t>
+  </si>
+  <si>
+    <t>Describe the task</t>
+  </si>
+  <si>
+    <t>Описание задачи</t>
+  </si>
+  <si>
+    <t>cases.compose.updateHint</t>
+  </si>
+  <si>
+    <t>What's new in the case?</t>
+  </si>
+  <si>
+    <t>Что нового по кейсу?</t>
+  </si>
+  <si>
+    <t>cases.compose.noteHint</t>
+  </si>
+  <si>
+    <t>Note (optional)</t>
+  </si>
+  <si>
+    <t>Заметка (необязательно)</t>
+  </si>
+  <si>
+    <t>cases.compose.fileNoteHint</t>
+  </si>
+  <si>
+    <t>What's in this file</t>
+  </si>
+  <si>
+    <t>Что на этом файле</t>
+  </si>
+  <si>
+    <t>cases.compose.checklist</t>
+  </si>
+  <si>
+    <t>Checklist item</t>
+  </si>
+  <si>
+    <t>Пункт списка</t>
+  </si>
+  <si>
+    <t>cases.compose.due</t>
+  </si>
+  <si>
+    <t>Due date</t>
+  </si>
+  <si>
+    <t>mine.tab.activeCases</t>
+  </si>
+  <si>
+    <t>Active cases</t>
+  </si>
+  <si>
+    <t>Активные дела</t>
+  </si>
+  <si>
+    <t>cases.tasks.dueOn</t>
+  </si>
+  <si>
+    <t>due {date}</t>
+  </si>
+  <si>
+    <t>cases.compose.remind</t>
+  </si>
+  <si>
+    <t>Reminder</t>
+  </si>
+  <si>
+    <t>Напоминание</t>
+  </si>
+  <si>
+    <t>cases.compose.attach</t>
+  </si>
+  <si>
+    <t>Attach</t>
+  </si>
+  <si>
+    <t>Прикрепить</t>
+  </si>
+  <si>
+    <t>cases.compose.photo</t>
+  </si>
+  <si>
+    <t>cases.compose.file</t>
+  </si>
+  <si>
+    <t>File</t>
+  </si>
+  <si>
+    <t>Файл</t>
+  </si>
+  <si>
+    <t>cases.compose.samplePhoto</t>
+  </si>
+  <si>
+    <t>Sample (photo)</t>
+  </si>
+  <si>
+    <t>Образец (фото)</t>
+  </si>
+  <si>
+    <t>cases.compose.sampleFile</t>
+  </si>
+  <si>
+    <t>Sample (file)</t>
+  </si>
+  <si>
+    <t>Образец (файл)</t>
+  </si>
+  <si>
+    <t>caseInvites.cancel</t>
+  </si>
+  <si>
+    <t>caseInvites.cancel.confirm</t>
+  </si>
+  <si>
+    <t>Cancel this invite?</t>
+  </si>
+  <si>
+    <t>Отменить приглашение?</t>
+  </si>
+  <si>
+    <t>caseInvites.cancelled</t>
+  </si>
+  <si>
+    <t>Invite cancelled</t>
+  </si>
+  <si>
+    <t>Приглашение отменено</t>
+  </si>
+  <si>
+    <t>caseInvites.reason</t>
+  </si>
+  <si>
+    <t>Reason: {reason}</t>
+  </si>
+  <si>
+    <t>Причина: {reason}</t>
+  </si>
+  <si>
+    <t>caseInvites.title</t>
+  </si>
+  <si>
+    <t>Invited attorneys</t>
+  </si>
+  <si>
+    <t>Приглашённые адвокаты</t>
+  </si>
+  <si>
+    <t>cases.accept.mismatchIntro</t>
+  </si>
+  <si>
+    <t>Please note:</t>
+  </si>
+  <si>
+    <t>Обратите внимание:</t>
+  </si>
+  <si>
+    <t>cases.accept.unverifiedLine</t>
+  </si>
+  <si>
+    <t>The attorney's license is not checked by LawBid — verify it with the state bar.</t>
+  </si>
+  <si>
+    <t>Лицензия адвоката не проверена LawBid — проверьте её в коллегии штата.</t>
+  </si>
+  <si>
+    <t>cases.contacts.notShared</t>
+  </si>
+  <si>
+    <t>The client's contacts are not available yet. Reopen the screen or contact support.</t>
+  </si>
+  <si>
+    <t>Контакты клиента пока не доступны. Откройте экран заново или обратитесь в поддержку.</t>
+  </si>
+  <si>
+    <t>cases.cover.auto</t>
+  </si>
+  <si>
+    <t>Auto</t>
+  </si>
+  <si>
+    <t>Авто</t>
+  </si>
+  <si>
+    <t>cases.cover.covers</t>
+  </si>
+  <si>
+    <t>Covers</t>
+  </si>
+  <si>
+    <t>Обложки</t>
+  </si>
+  <si>
+    <t>cases.cover.iconOption</t>
+  </si>
+  <si>
+    <t>Icon {n}</t>
+  </si>
+  <si>
+    <t>Иконка {n}</t>
+  </si>
+  <si>
+    <t>cases.cover.icons</t>
+  </si>
+  <si>
+    <t>Icons</t>
+  </si>
+  <si>
+    <t>Иконки</t>
+  </si>
+  <si>
+    <t>cases.cover.option</t>
+  </si>
+  <si>
+    <t>Cover {n}</t>
+  </si>
+  <si>
+    <t>Обложка {n}</t>
+  </si>
+  <si>
+    <t>cases.cover.subtitle</t>
+  </si>
+  <si>
+    <t>Attorneys see this picture instead of your photo. Your photos stay hidden until you accept a bid.</t>
+  </si>
+  <si>
+    <t>Адвокаты видят эту картинку вместо вашего фото. Ваши фото скрыты, пока вы не примете ставку.</t>
+  </si>
+  <si>
+    <t>cases.cover.title</t>
+  </si>
+  <si>
+    <t>Card cover</t>
+  </si>
+  <si>
+    <t>Обложка карточки</t>
+  </si>
+  <si>
+    <t>cases.create.urgency.title</t>
+  </si>
+  <si>
+    <t>How soon do you need an attorney?</t>
+  </si>
+  <si>
+    <t>Как скоро нужен адвокат?</t>
+  </si>
+  <si>
+    <t>cases.facts.budget</t>
+  </si>
+  <si>
+    <t>Budget</t>
+  </si>
+  <si>
+    <t>Бюджет</t>
+  </si>
+  <si>
+    <t>cases.facts.negotiable</t>
+  </si>
+  <si>
+    <t>Negotiable</t>
+  </si>
+  <si>
+    <t>Обсуждается</t>
+  </si>
+  <si>
+    <t>cases.facts.notSet</t>
+  </si>
+  <si>
+    <t>Not set</t>
+  </si>
+  <si>
+    <t>Не указано</t>
+  </si>
+  <si>
+    <t>cases.facts.state</t>
+  </si>
+  <si>
+    <t>cases.facts.urgency</t>
+  </si>
+  <si>
+    <t>Urgency</t>
+  </si>
+  <si>
+    <t>Срочность</t>
+  </si>
+  <si>
+    <t>cases.field.urgency</t>
+  </si>
+  <si>
+    <t>cases.mine.archived</t>
+  </si>
+  <si>
+    <t>Archive</t>
+  </si>
+  <si>
+    <t>Архив</t>
+  </si>
+  <si>
+    <t>cases.mine.finished</t>
+  </si>
+  <si>
+    <t>Finished</t>
+  </si>
+  <si>
+    <t>Закрытые</t>
+  </si>
+  <si>
+    <t>cases.outsideStates.attorney</t>
+  </si>
+  <si>
+    <t>You have no license in this case's state. You can still bid: the client will see the states you're licensed in.</t>
+  </si>
+  <si>
+    <t>У вас нет лицензии в штате этого кейса. Отклик отправить можно: клиент увидит, в каких штатах вы лицензированы.</t>
+  </si>
+  <si>
+    <t>cases.outsideStates.client</t>
+  </si>
+  <si>
+    <t>The attorney is licensed in: {states}. This case's state isn't one of them. Ask how they'll handle it.</t>
+  </si>
+  <si>
+    <t>Адвокат лицензирован в: {states}. Штата этого кейса среди них нет. Уточните, как будет вестись дело.</t>
+  </si>
+  <si>
+    <t>cases.outsideStates.clientNoList</t>
+  </si>
+  <si>
+    <t>The attorney has no license in this case's state. Ask how they'll handle it.</t>
+  </si>
+  <si>
+    <t>У адвоката нет лицензии в штате этого кейса. Уточните, как будет вестись дело.</t>
+  </si>
+  <si>
+    <t>cases.overview.meta</t>
+  </si>
+  <si>
+    <t>Published {published} · Accepted {accepted} · {bids} bids</t>
+  </si>
+  <si>
+    <t>Опубликован {published} · Принят {accepted} · Бидов: {bids}</t>
+  </si>
+  <si>
+    <t>cases.owner.closeShort</t>
+  </si>
+  <si>
+    <t>cases.owner.keepAliveShort</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Да</t>
+  </si>
+  <si>
+    <t>cases.owner.keptAlive</t>
+  </si>
+  <si>
+    <t>Your case stays open</t>
+  </si>
+  <si>
+    <t>Кейс остаётся открытым</t>
+  </si>
+  <si>
+    <t>cases.owner.staleShort</t>
+  </si>
+  <si>
+    <t>Still relevant?</t>
+  </si>
+  <si>
+    <t>Кейс ещё актуален?</t>
+  </si>
+  <si>
+    <t>cases.photos.failedHint</t>
+  </si>
+  <si>
+    <t>Retry or remove the file that failed to upload.</t>
+  </si>
+  <si>
+    <t>Повторите или удалите файл, который не загрузился.</t>
+  </si>
+  <si>
+    <t>cases.urgency.flexible</t>
+  </si>
+  <si>
+    <t>No rush</t>
+  </si>
+  <si>
+    <t>Не срочно</t>
+  </si>
+  <si>
+    <t>cases.urgency.soon</t>
+  </si>
+  <si>
+    <t>This week</t>
+  </si>
+  <si>
+    <t>На этой неделе</t>
+  </si>
+  <si>
+    <t>cases.urgency.urgent</t>
+  </si>
+  <si>
+    <t>Urgent</t>
+  </si>
+  <si>
+    <t>Срочно</t>
+  </si>
+  <si>
+    <t>invite.mismatch.practice</t>
+  </si>
+  <si>
+    <t>This case is outside the attorney's practice areas.</t>
+  </si>
+  <si>
+    <t>Дело не в практиках этого адвоката.</t>
+  </si>
+  <si>
+    <t>invite.mismatch.state</t>
+  </si>
+  <si>
+    <t>This attorney has no licence in the case's state.</t>
+  </si>
+  <si>
+    <t>У адвоката нет лицензии в штате этого дела.</t>
+  </si>
+  <si>
+    <t>invite.offer.alreadyBid</t>
+  </si>
+  <si>
+    <t>This attorney already sent a bid on this case.</t>
+  </si>
+  <si>
+    <t>Этот адвокат уже прислал бид на это дело.</t>
+  </si>
+  <si>
+    <t>invite.offer.body</t>
+  </si>
+  <si>
+    <t>The attorney sees the case and answers with a bid or declines. Your name and contacts stay hidden until you accept a bid.</t>
+  </si>
+  <si>
+    <t>Адвокат увидит дело и ответит бидом или откажется. Ваше имя и контакты скрыты, пока вы не примете бид.</t>
+  </si>
+  <si>
+    <t>invite.offer.budgetHint</t>
+  </si>
+  <si>
+    <t>invite.offer.createCase</t>
+  </si>
+  <si>
+    <t>Create a case</t>
+  </si>
+  <si>
+    <t>Создать дело</t>
+  </si>
+  <si>
+    <t>invite.offer.message</t>
+  </si>
+  <si>
+    <t>Note to the attorney</t>
+  </si>
+  <si>
+    <t>Сообщение адвокату</t>
+  </si>
+  <si>
+    <t>invite.offer.messageHint</t>
+  </si>
+  <si>
+    <t>Optional. No phone numbers or emails.</t>
+  </si>
+  <si>
+    <t>Необязательно. Без телефонов и email.</t>
+  </si>
+  <si>
+    <t>invite.offer.noCases</t>
+  </si>
+  <si>
+    <t>You have no open cases. Create one, then offer it to the attorney.</t>
+  </si>
+  <si>
+    <t>У вас нет открытых дел. Создайте дело, а потом предложите его адвокату.</t>
+  </si>
+  <si>
+    <t>invite.offer.pickCase</t>
+  </si>
+  <si>
+    <t>Which case?</t>
+  </si>
+  <si>
+    <t>Какое дело?</t>
+  </si>
+  <si>
+    <t>invite.offer.send</t>
+  </si>
+  <si>
+    <t>invite.offer.sent</t>
+  </si>
+  <si>
+    <t>Sent. We'll let you know when the attorney answers.</t>
+  </si>
+  <si>
+    <t>Отправлено. Мы сообщим, когда адвокат ответит.</t>
+  </si>
+  <si>
+    <t>invite.offer.title</t>
+  </si>
+  <si>
+    <t>Offer a case to {name}</t>
+  </si>
+  <si>
+    <t>Предложить дело: {name}</t>
+  </si>
+  <si>
+    <t>invites.answer</t>
+  </si>
+  <si>
+    <t>Answer with a bid</t>
+  </si>
+  <si>
+    <t>Ответить бидом</t>
+  </si>
+  <si>
+    <t>invites.budget</t>
+  </si>
+  <si>
+    <t>Client's budget: {amount}</t>
+  </si>
+  <si>
+    <t>Бюджет клиента: {amount}</t>
+  </si>
+  <si>
+    <t>invites.clientNote</t>
+  </si>
+  <si>
+    <t>Client's note</t>
+  </si>
+  <si>
+    <t>Сообщение клиента</t>
+  </si>
+  <si>
+    <t>invites.decline</t>
+  </si>
+  <si>
+    <t>Decline</t>
+  </si>
+  <si>
+    <t>Отказаться</t>
+  </si>
+  <si>
+    <t>invites.decline.confirm</t>
+  </si>
+  <si>
+    <t>invites.decline.reason</t>
+  </si>
+  <si>
+    <t>Reason (optional, the client sees it)</t>
+  </si>
+  <si>
+    <t>Причина (необязательно, клиент её увидит)</t>
+  </si>
+  <si>
+    <t>invites.decline.title</t>
+  </si>
+  <si>
+    <t>Decline the case?</t>
+  </si>
+  <si>
+    <t>Отказаться от дела?</t>
+  </si>
+  <si>
+    <t>invites.declined</t>
+  </si>
+  <si>
+    <t>Declined. The client was told.</t>
+  </si>
+  <si>
+    <t>Вы отказались. Клиент получил уведомление.</t>
+  </si>
+  <si>
+    <t>invites.empty</t>
+  </si>
+  <si>
+    <t>No invitations yet</t>
+  </si>
+  <si>
+    <t>Пока нет приглашений</t>
+  </si>
+  <si>
+    <t>invites.empty.body</t>
+  </si>
+  <si>
+    <t>When a client offers you a case, it appears here.</t>
+  </si>
+  <si>
+    <t>Когда клиент предложит вам дело, оно появится здесь.</t>
+  </si>
+  <si>
+    <t>invites.expires</t>
+  </si>
+  <si>
+    <t>Answer by {date}</t>
+  </si>
+  <si>
+    <t>Ответить до {date}</t>
+  </si>
+  <si>
+    <t>invites.noBudget</t>
+  </si>
+  <si>
+    <t>Budget to discuss</t>
+  </si>
+  <si>
+    <t>Бюджет обсуждается</t>
+  </si>
+  <si>
+    <t>invites.open</t>
+  </si>
+  <si>
+    <t>Open case</t>
+  </si>
+  <si>
+    <t>Открыть дело</t>
+  </si>
+  <si>
+    <t>invites.section</t>
+  </si>
+  <si>
+    <t>Invitations</t>
+  </si>
+  <si>
+    <t>Приглашения</t>
+  </si>
+  <si>
+    <t>invites.title</t>
+  </si>
+  <si>
+    <t>Invitations from clients</t>
+  </si>
+  <si>
+    <t>Приглашения от клиентов</t>
+  </si>
+  <si>
+    <t>invite.offer.budget</t>
+  </si>
+  <si>
+    <t>Your budget, $</t>
+  </si>
+  <si>
+    <t>Ваш бюджет, $</t>
+  </si>
+  <si>
+    <t>cases.files.count.few</t>
+  </si>
+  <si>
+    <t>cases.files.count.many</t>
+  </si>
+  <si>
+    <t>{count} файлов</t>
   </si>
 </sst>
 </file>
@@ -6654,7 +7920,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C751"/>
+  <dimension ref="A1:C904"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -14922,6 +16188,1689 @@
         <v>2088</v>
       </c>
     </row>
+    <row r="752" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A752" t="s">
+        <v>2089</v>
+      </c>
+      <c r="B752" t="s">
+        <v>2090</v>
+      </c>
+      <c r="C752" t="s">
+        <v>2091</v>
+      </c>
+    </row>
+    <row r="753" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A753" t="s">
+        <v>2092</v>
+      </c>
+      <c r="B753" t="s">
+        <v>2093</v>
+      </c>
+      <c r="C753" t="s">
+        <v>2094</v>
+      </c>
+    </row>
+    <row r="754" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A754" t="s">
+        <v>2095</v>
+      </c>
+      <c r="B754" t="s">
+        <v>90</v>
+      </c>
+      <c r="C754" t="s">
+        <v>2096</v>
+      </c>
+    </row>
+    <row r="755" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A755" t="s">
+        <v>2097</v>
+      </c>
+      <c r="B755" t="s">
+        <v>2098</v>
+      </c>
+      <c r="C755" t="s">
+        <v>2099</v>
+      </c>
+    </row>
+    <row r="756" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A756" t="s">
+        <v>2100</v>
+      </c>
+      <c r="B756" t="s">
+        <v>2101</v>
+      </c>
+      <c r="C756" t="s">
+        <v>2102</v>
+      </c>
+    </row>
+    <row r="757" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A757" t="s">
+        <v>2103</v>
+      </c>
+      <c r="B757" t="s">
+        <v>2104</v>
+      </c>
+      <c r="C757" t="s">
+        <v>2105</v>
+      </c>
+    </row>
+    <row r="758" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A758" t="s">
+        <v>2106</v>
+      </c>
+      <c r="B758" t="s">
+        <v>2107</v>
+      </c>
+      <c r="C758" t="s">
+        <v>2108</v>
+      </c>
+    </row>
+    <row r="759" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A759" t="s">
+        <v>2109</v>
+      </c>
+      <c r="B759" t="s">
+        <v>2110</v>
+      </c>
+      <c r="C759" t="s">
+        <v>2111</v>
+      </c>
+    </row>
+    <row r="760" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A760" t="s">
+        <v>2112</v>
+      </c>
+      <c r="B760" t="s">
+        <v>2113</v>
+      </c>
+      <c r="C760" t="s">
+        <v>2114</v>
+      </c>
+    </row>
+    <row r="761" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A761" t="s">
+        <v>2115</v>
+      </c>
+      <c r="B761" t="s">
+        <v>2116</v>
+      </c>
+      <c r="C761" t="s">
+        <v>2117</v>
+      </c>
+    </row>
+    <row r="762" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A762" t="s">
+        <v>2118</v>
+      </c>
+      <c r="B762" t="s">
+        <v>2119</v>
+      </c>
+      <c r="C762" t="s">
+        <v>2120</v>
+      </c>
+    </row>
+    <row r="763" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A763" t="s">
+        <v>2121</v>
+      </c>
+      <c r="B763" t="s">
+        <v>2122</v>
+      </c>
+      <c r="C763" t="s">
+        <v>2123</v>
+      </c>
+    </row>
+    <row r="764" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A764" t="s">
+        <v>2124</v>
+      </c>
+      <c r="B764" t="s">
+        <v>970</v>
+      </c>
+      <c r="C764" t="s">
+        <v>971</v>
+      </c>
+    </row>
+    <row r="765" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A765" t="s">
+        <v>2125</v>
+      </c>
+      <c r="B765" t="s">
+        <v>2126</v>
+      </c>
+      <c r="C765" t="s">
+        <v>2127</v>
+      </c>
+    </row>
+    <row r="766" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A766" t="s">
+        <v>2128</v>
+      </c>
+      <c r="B766" t="s">
+        <v>2129</v>
+      </c>
+      <c r="C766" t="s">
+        <v>2130</v>
+      </c>
+    </row>
+    <row r="767" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A767" t="s">
+        <v>2131</v>
+      </c>
+      <c r="B767" t="s">
+        <v>2132</v>
+      </c>
+      <c r="C767" t="s">
+        <v>2133</v>
+      </c>
+    </row>
+    <row r="768" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A768" t="s">
+        <v>2134</v>
+      </c>
+      <c r="B768" t="s">
+        <v>2135</v>
+      </c>
+      <c r="C768" t="s">
+        <v>2136</v>
+      </c>
+    </row>
+    <row r="769" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A769" t="s">
+        <v>2137</v>
+      </c>
+      <c r="B769" t="s">
+        <v>2138</v>
+      </c>
+      <c r="C769" t="s">
+        <v>2139</v>
+      </c>
+    </row>
+    <row r="770" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A770" t="s">
+        <v>2140</v>
+      </c>
+      <c r="B770" t="s">
+        <v>2141</v>
+      </c>
+      <c r="C770" t="s">
+        <v>2142</v>
+      </c>
+    </row>
+    <row r="771" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A771" t="s">
+        <v>2143</v>
+      </c>
+      <c r="B771" t="s">
+        <v>2144</v>
+      </c>
+      <c r="C771" t="s">
+        <v>2127</v>
+      </c>
+    </row>
+    <row r="772" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A772" t="s">
+        <v>2145</v>
+      </c>
+      <c r="B772" t="s">
+        <v>2146</v>
+      </c>
+      <c r="C772" t="s">
+        <v>2147</v>
+      </c>
+    </row>
+    <row r="773" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A773" t="s">
+        <v>2148</v>
+      </c>
+      <c r="B773" t="s">
+        <v>2149</v>
+      </c>
+      <c r="C773" t="s">
+        <v>2150</v>
+      </c>
+    </row>
+    <row r="774" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A774" t="s">
+        <v>2151</v>
+      </c>
+      <c r="B774" t="s">
+        <v>2152</v>
+      </c>
+      <c r="C774" t="s">
+        <v>2153</v>
+      </c>
+    </row>
+    <row r="775" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A775" t="s">
+        <v>2154</v>
+      </c>
+      <c r="B775" t="s">
+        <v>2155</v>
+      </c>
+      <c r="C775" t="s">
+        <v>2156</v>
+      </c>
+    </row>
+    <row r="776" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A776" t="s">
+        <v>2157</v>
+      </c>
+      <c r="B776" t="s">
+        <v>2158</v>
+      </c>
+      <c r="C776" t="s">
+        <v>2159</v>
+      </c>
+    </row>
+    <row r="777" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A777" t="s">
+        <v>2160</v>
+      </c>
+      <c r="B777" t="s">
+        <v>2161</v>
+      </c>
+      <c r="C777" t="s">
+        <v>2162</v>
+      </c>
+    </row>
+    <row r="778" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A778" t="s">
+        <v>2163</v>
+      </c>
+      <c r="B778" t="s">
+        <v>2164</v>
+      </c>
+      <c r="C778" t="s">
+        <v>2165</v>
+      </c>
+    </row>
+    <row r="779" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A779" t="s">
+        <v>2166</v>
+      </c>
+      <c r="B779" t="s">
+        <v>2167</v>
+      </c>
+      <c r="C779" t="s">
+        <v>2168</v>
+      </c>
+    </row>
+    <row r="780" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A780" t="s">
+        <v>2169</v>
+      </c>
+      <c r="B780" t="s">
+        <v>270</v>
+      </c>
+      <c r="C780" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="781" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A781" t="s">
+        <v>2170</v>
+      </c>
+      <c r="B781" t="s">
+        <v>2171</v>
+      </c>
+      <c r="C781" t="s">
+        <v>2172</v>
+      </c>
+    </row>
+    <row r="782" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A782" t="s">
+        <v>2173</v>
+      </c>
+      <c r="B782" t="s">
+        <v>2174</v>
+      </c>
+      <c r="C782" t="s">
+        <v>2175</v>
+      </c>
+    </row>
+    <row r="783" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A783" t="s">
+        <v>2176</v>
+      </c>
+      <c r="B783" t="s">
+        <v>2177</v>
+      </c>
+      <c r="C783" t="s">
+        <v>2178</v>
+      </c>
+    </row>
+    <row r="784" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A784" t="s">
+        <v>2179</v>
+      </c>
+      <c r="B784" t="s">
+        <v>2180</v>
+      </c>
+      <c r="C784" t="s">
+        <v>2181</v>
+      </c>
+    </row>
+    <row r="785" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A785" t="s">
+        <v>2182</v>
+      </c>
+      <c r="B785" t="s">
+        <v>2183</v>
+      </c>
+      <c r="C785" t="s">
+        <v>2184</v>
+      </c>
+    </row>
+    <row r="786" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A786" t="s">
+        <v>2185</v>
+      </c>
+      <c r="B786" t="s">
+        <v>2186</v>
+      </c>
+      <c r="C786" t="s">
+        <v>2187</v>
+      </c>
+    </row>
+    <row r="787" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A787" t="s">
+        <v>2188</v>
+      </c>
+      <c r="B787" t="s">
+        <v>2189</v>
+      </c>
+      <c r="C787" t="s">
+        <v>2190</v>
+      </c>
+    </row>
+    <row r="788" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A788" t="s">
+        <v>2191</v>
+      </c>
+      <c r="B788" t="s">
+        <v>2192</v>
+      </c>
+      <c r="C788" t="s">
+        <v>2193</v>
+      </c>
+    </row>
+    <row r="789" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A789" t="s">
+        <v>2194</v>
+      </c>
+      <c r="B789" t="s">
+        <v>2195</v>
+      </c>
+      <c r="C789" t="s">
+        <v>2196</v>
+      </c>
+    </row>
+    <row r="790" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A790" t="s">
+        <v>2197</v>
+      </c>
+      <c r="B790" t="s">
+        <v>2198</v>
+      </c>
+      <c r="C790" t="s">
+        <v>2199</v>
+      </c>
+    </row>
+    <row r="791" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A791" t="s">
+        <v>2200</v>
+      </c>
+      <c r="B791" t="s">
+        <v>2201</v>
+      </c>
+      <c r="C791" t="s">
+        <v>2202</v>
+      </c>
+    </row>
+    <row r="792" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A792" t="s">
+        <v>2203</v>
+      </c>
+      <c r="B792" t="s">
+        <v>2204</v>
+      </c>
+      <c r="C792" t="s">
+        <v>2205</v>
+      </c>
+    </row>
+    <row r="793" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A793" t="s">
+        <v>2206</v>
+      </c>
+      <c r="B793" t="s">
+        <v>2207</v>
+      </c>
+      <c r="C793" t="s">
+        <v>2208</v>
+      </c>
+    </row>
+    <row r="794" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A794" t="s">
+        <v>2209</v>
+      </c>
+      <c r="B794" t="s">
+        <v>2210</v>
+      </c>
+      <c r="C794" t="s">
+        <v>2211</v>
+      </c>
+    </row>
+    <row r="795" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A795" t="s">
+        <v>2212</v>
+      </c>
+      <c r="B795" t="s">
+        <v>2213</v>
+      </c>
+      <c r="C795" t="s">
+        <v>2214</v>
+      </c>
+    </row>
+    <row r="796" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A796" t="s">
+        <v>2215</v>
+      </c>
+      <c r="B796" t="s">
+        <v>2216</v>
+      </c>
+      <c r="C796" t="s">
+        <v>2217</v>
+      </c>
+    </row>
+    <row r="797" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A797" t="s">
+        <v>2218</v>
+      </c>
+      <c r="B797" t="s">
+        <v>2219</v>
+      </c>
+      <c r="C797" t="s">
+        <v>2220</v>
+      </c>
+    </row>
+    <row r="798" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A798" t="s">
+        <v>2221</v>
+      </c>
+      <c r="B798" t="s">
+        <v>2222</v>
+      </c>
+      <c r="C798" t="s">
+        <v>2223</v>
+      </c>
+    </row>
+    <row r="799" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A799" t="s">
+        <v>2224</v>
+      </c>
+      <c r="B799" t="s">
+        <v>2225</v>
+      </c>
+      <c r="C799" t="s">
+        <v>2226</v>
+      </c>
+    </row>
+    <row r="800" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A800" t="s">
+        <v>2227</v>
+      </c>
+      <c r="B800" t="s">
+        <v>2228</v>
+      </c>
+      <c r="C800" t="s">
+        <v>2229</v>
+      </c>
+    </row>
+    <row r="801" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A801" t="s">
+        <v>2230</v>
+      </c>
+      <c r="B801" t="s">
+        <v>2231</v>
+      </c>
+      <c r="C801" t="s">
+        <v>2232</v>
+      </c>
+    </row>
+    <row r="802" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A802" t="s">
+        <v>2233</v>
+      </c>
+      <c r="B802" t="s">
+        <v>2234</v>
+      </c>
+      <c r="C802" t="s">
+        <v>2235</v>
+      </c>
+    </row>
+    <row r="803" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A803" t="s">
+        <v>2236</v>
+      </c>
+      <c r="B803" t="s">
+        <v>2237</v>
+      </c>
+      <c r="C803" t="s">
+        <v>2238</v>
+      </c>
+    </row>
+    <row r="804" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A804" t="s">
+        <v>2239</v>
+      </c>
+      <c r="B804" t="s">
+        <v>220</v>
+      </c>
+      <c r="C804" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="805" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A805" t="s">
+        <v>2240</v>
+      </c>
+      <c r="B805" t="s">
+        <v>2241</v>
+      </c>
+      <c r="C805" t="s">
+        <v>2242</v>
+      </c>
+    </row>
+    <row r="806" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A806" t="s">
+        <v>2243</v>
+      </c>
+      <c r="B806" t="s">
+        <v>2244</v>
+      </c>
+      <c r="C806" t="s">
+        <v>2245</v>
+      </c>
+    </row>
+    <row r="807" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A807" t="s">
+        <v>2246</v>
+      </c>
+      <c r="B807" t="s">
+        <v>2247</v>
+      </c>
+      <c r="C807" t="s">
+        <v>2248</v>
+      </c>
+    </row>
+    <row r="808" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A808" t="s">
+        <v>2249</v>
+      </c>
+      <c r="B808" t="s">
+        <v>2250</v>
+      </c>
+      <c r="C808" t="s">
+        <v>2251</v>
+      </c>
+    </row>
+    <row r="809" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A809" t="s">
+        <v>2252</v>
+      </c>
+      <c r="B809" t="s">
+        <v>2253</v>
+      </c>
+      <c r="C809" t="s">
+        <v>2254</v>
+      </c>
+    </row>
+    <row r="810" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A810" t="s">
+        <v>2255</v>
+      </c>
+      <c r="B810" t="s">
+        <v>2256</v>
+      </c>
+      <c r="C810" t="s">
+        <v>2257</v>
+      </c>
+    </row>
+    <row r="811" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A811" t="s">
+        <v>2258</v>
+      </c>
+      <c r="B811" t="s">
+        <v>2259</v>
+      </c>
+      <c r="C811" t="s">
+        <v>2260</v>
+      </c>
+    </row>
+    <row r="812" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A812" t="s">
+        <v>2261</v>
+      </c>
+      <c r="B812" t="s">
+        <v>2262</v>
+      </c>
+      <c r="C812" t="s">
+        <v>2263</v>
+      </c>
+    </row>
+    <row r="813" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A813" t="s">
+        <v>2264</v>
+      </c>
+      <c r="B813" t="s">
+        <v>356</v>
+      </c>
+      <c r="C813" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="814" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A814" t="s">
+        <v>2265</v>
+      </c>
+      <c r="B814" t="s">
+        <v>2266</v>
+      </c>
+      <c r="C814" t="s">
+        <v>2267</v>
+      </c>
+    </row>
+    <row r="815" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A815" t="s">
+        <v>2268</v>
+      </c>
+      <c r="B815" t="s">
+        <v>2269</v>
+      </c>
+      <c r="C815" t="s">
+        <v>2270</v>
+      </c>
+    </row>
+    <row r="816" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A816" t="s">
+        <v>2271</v>
+      </c>
+      <c r="B816" t="s">
+        <v>344</v>
+      </c>
+      <c r="C816" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="817" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A817" t="s">
+        <v>2272</v>
+      </c>
+      <c r="B817" t="s">
+        <v>2273</v>
+      </c>
+      <c r="C817" t="s">
+        <v>2274</v>
+      </c>
+    </row>
+    <row r="818" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A818" t="s">
+        <v>2275</v>
+      </c>
+      <c r="B818" t="s">
+        <v>2276</v>
+      </c>
+      <c r="C818" t="s">
+        <v>2277</v>
+      </c>
+    </row>
+    <row r="819" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A819" t="s">
+        <v>2278</v>
+      </c>
+      <c r="B819" t="s">
+        <v>2279</v>
+      </c>
+      <c r="C819" t="s">
+        <v>2280</v>
+      </c>
+    </row>
+    <row r="820" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A820" t="s">
+        <v>2281</v>
+      </c>
+      <c r="B820" t="s">
+        <v>2259</v>
+      </c>
+      <c r="C820" t="s">
+        <v>2260</v>
+      </c>
+    </row>
+    <row r="821" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A821" t="s">
+        <v>2282</v>
+      </c>
+      <c r="B821" t="s">
+        <v>100</v>
+      </c>
+      <c r="C821" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="822" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A822" t="s">
+        <v>2283</v>
+      </c>
+      <c r="B822" t="s">
+        <v>2284</v>
+      </c>
+      <c r="C822" t="s">
+        <v>2285</v>
+      </c>
+    </row>
+    <row r="823" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A823" t="s">
+        <v>2286</v>
+      </c>
+      <c r="B823" t="s">
+        <v>2287</v>
+      </c>
+      <c r="C823" t="s">
+        <v>2288</v>
+      </c>
+    </row>
+    <row r="824" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A824" t="s">
+        <v>2289</v>
+      </c>
+      <c r="B824" t="s">
+        <v>2290</v>
+      </c>
+      <c r="C824" t="s">
+        <v>2291</v>
+      </c>
+    </row>
+    <row r="825" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A825" t="s">
+        <v>2292</v>
+      </c>
+      <c r="B825" t="s">
+        <v>2293</v>
+      </c>
+      <c r="C825" t="s">
+        <v>2294</v>
+      </c>
+    </row>
+    <row r="826" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A826" t="s">
+        <v>2295</v>
+      </c>
+      <c r="B826" t="s">
+        <v>2296</v>
+      </c>
+      <c r="C826" t="s">
+        <v>2297</v>
+      </c>
+    </row>
+    <row r="827" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A827" t="s">
+        <v>2298</v>
+      </c>
+      <c r="B827" t="s">
+        <v>2299</v>
+      </c>
+      <c r="C827" t="s">
+        <v>2300</v>
+      </c>
+    </row>
+    <row r="828" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A828" t="s">
+        <v>2301</v>
+      </c>
+      <c r="B828" t="s">
+        <v>2302</v>
+      </c>
+      <c r="C828" t="s">
+        <v>2303</v>
+      </c>
+    </row>
+    <row r="829" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A829" t="s">
+        <v>2304</v>
+      </c>
+      <c r="B829" t="s">
+        <v>2305</v>
+      </c>
+      <c r="C829" t="s">
+        <v>2091</v>
+      </c>
+    </row>
+    <row r="830" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A830" t="s">
+        <v>2306</v>
+      </c>
+      <c r="B830" t="s">
+        <v>2307</v>
+      </c>
+      <c r="C830" t="s">
+        <v>2308</v>
+      </c>
+    </row>
+    <row r="831" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A831" t="s">
+        <v>2309</v>
+      </c>
+      <c r="B831" t="s">
+        <v>2310</v>
+      </c>
+      <c r="C831" t="s">
+        <v>1598</v>
+      </c>
+    </row>
+    <row r="832" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A832" t="s">
+        <v>2311</v>
+      </c>
+      <c r="B832" t="s">
+        <v>2312</v>
+      </c>
+      <c r="C832" t="s">
+        <v>2313</v>
+      </c>
+    </row>
+    <row r="833" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A833" t="s">
+        <v>2314</v>
+      </c>
+      <c r="B833" t="s">
+        <v>2315</v>
+      </c>
+      <c r="C833" t="s">
+        <v>2316</v>
+      </c>
+    </row>
+    <row r="834" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A834" t="s">
+        <v>2317</v>
+      </c>
+      <c r="B834" t="s">
+        <v>2144</v>
+      </c>
+      <c r="C834" t="s">
+        <v>2127</v>
+      </c>
+    </row>
+    <row r="835" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A835" t="s">
+        <v>2318</v>
+      </c>
+      <c r="B835" t="s">
+        <v>2319</v>
+      </c>
+      <c r="C835" t="s">
+        <v>2320</v>
+      </c>
+    </row>
+    <row r="836" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A836" t="s">
+        <v>2321</v>
+      </c>
+      <c r="B836" t="s">
+        <v>2322</v>
+      </c>
+      <c r="C836" t="s">
+        <v>2323</v>
+      </c>
+    </row>
+    <row r="837" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A837" t="s">
+        <v>2324</v>
+      </c>
+      <c r="B837" t="s">
+        <v>2325</v>
+      </c>
+      <c r="C837" t="s">
+        <v>2326</v>
+      </c>
+    </row>
+    <row r="838" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A838" t="s">
+        <v>2327</v>
+      </c>
+      <c r="B838" t="s">
+        <v>95</v>
+      </c>
+      <c r="C838" t="s">
+        <v>1989</v>
+      </c>
+    </row>
+    <row r="839" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A839" t="s">
+        <v>2328</v>
+      </c>
+      <c r="B839" t="s">
+        <v>2329</v>
+      </c>
+      <c r="C839" t="s">
+        <v>2330</v>
+      </c>
+    </row>
+    <row r="840" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A840" t="s">
+        <v>2331</v>
+      </c>
+      <c r="B840" t="s">
+        <v>2332</v>
+      </c>
+      <c r="C840" t="s">
+        <v>2333</v>
+      </c>
+    </row>
+    <row r="841" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A841" t="s">
+        <v>2334</v>
+      </c>
+      <c r="B841" t="s">
+        <v>2335</v>
+      </c>
+      <c r="C841" t="s">
+        <v>2336</v>
+      </c>
+    </row>
+    <row r="842" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A842" t="s">
+        <v>2337</v>
+      </c>
+      <c r="B842" t="s">
+        <v>2338</v>
+      </c>
+      <c r="C842" t="s">
+        <v>2339</v>
+      </c>
+    </row>
+    <row r="843" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A843" t="s">
+        <v>2340</v>
+      </c>
+      <c r="B843" t="s">
+        <v>2341</v>
+      </c>
+      <c r="C843" t="s">
+        <v>2342</v>
+      </c>
+    </row>
+    <row r="844" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A844" t="s">
+        <v>2343</v>
+      </c>
+      <c r="B844" t="s">
+        <v>2344</v>
+      </c>
+      <c r="C844" t="s">
+        <v>2345</v>
+      </c>
+    </row>
+    <row r="845" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A845" t="s">
+        <v>2346</v>
+      </c>
+      <c r="B845" t="s">
+        <v>2347</v>
+      </c>
+      <c r="C845" t="s">
+        <v>2348</v>
+      </c>
+    </row>
+    <row r="846" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A846" t="s">
+        <v>2349</v>
+      </c>
+      <c r="B846" t="s">
+        <v>2350</v>
+      </c>
+      <c r="C846" t="s">
+        <v>2351</v>
+      </c>
+    </row>
+    <row r="847" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A847" t="s">
+        <v>2352</v>
+      </c>
+      <c r="B847" t="s">
+        <v>2353</v>
+      </c>
+      <c r="C847" t="s">
+        <v>2354</v>
+      </c>
+    </row>
+    <row r="848" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A848" t="s">
+        <v>2355</v>
+      </c>
+      <c r="B848" t="s">
+        <v>2356</v>
+      </c>
+      <c r="C848" t="s">
+        <v>2357</v>
+      </c>
+    </row>
+    <row r="849" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A849" t="s">
+        <v>2358</v>
+      </c>
+      <c r="B849" t="s">
+        <v>2359</v>
+      </c>
+      <c r="C849" t="s">
+        <v>2360</v>
+      </c>
+    </row>
+    <row r="850" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A850" t="s">
+        <v>2361</v>
+      </c>
+      <c r="B850" t="s">
+        <v>2362</v>
+      </c>
+      <c r="C850" t="s">
+        <v>2363</v>
+      </c>
+    </row>
+    <row r="851" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A851" t="s">
+        <v>2364</v>
+      </c>
+      <c r="B851" t="s">
+        <v>2365</v>
+      </c>
+      <c r="C851" t="s">
+        <v>2366</v>
+      </c>
+    </row>
+    <row r="852" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A852" t="s">
+        <v>2367</v>
+      </c>
+      <c r="B852" t="s">
+        <v>2368</v>
+      </c>
+      <c r="C852" t="s">
+        <v>2369</v>
+      </c>
+    </row>
+    <row r="853" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A853" t="s">
+        <v>2370</v>
+      </c>
+      <c r="B853" t="s">
+        <v>2371</v>
+      </c>
+      <c r="C853" t="s">
+        <v>2372</v>
+      </c>
+    </row>
+    <row r="854" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A854" t="s">
+        <v>2373</v>
+      </c>
+      <c r="B854" t="s">
+        <v>2374</v>
+      </c>
+      <c r="C854" t="s">
+        <v>2375</v>
+      </c>
+    </row>
+    <row r="855" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A855" t="s">
+        <v>2376</v>
+      </c>
+      <c r="B855" t="s">
+        <v>2377</v>
+      </c>
+      <c r="C855" t="s">
+        <v>2378</v>
+      </c>
+    </row>
+    <row r="856" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A856" t="s">
+        <v>2379</v>
+      </c>
+      <c r="B856" t="s">
+        <v>2380</v>
+      </c>
+      <c r="C856" t="s">
+        <v>2381</v>
+      </c>
+    </row>
+    <row r="857" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A857" t="s">
+        <v>2382</v>
+      </c>
+      <c r="B857" t="s">
+        <v>1564</v>
+      </c>
+      <c r="C857" t="s">
+        <v>1565</v>
+      </c>
+    </row>
+    <row r="858" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A858" t="s">
+        <v>2383</v>
+      </c>
+      <c r="B858" t="s">
+        <v>2384</v>
+      </c>
+      <c r="C858" t="s">
+        <v>2385</v>
+      </c>
+    </row>
+    <row r="859" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A859" t="s">
+        <v>2386</v>
+      </c>
+      <c r="B859" t="s">
+        <v>2384</v>
+      </c>
+      <c r="C859" t="s">
+        <v>2385</v>
+      </c>
+    </row>
+    <row r="860" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A860" t="s">
+        <v>2387</v>
+      </c>
+      <c r="B860" t="s">
+        <v>2388</v>
+      </c>
+      <c r="C860" t="s">
+        <v>2389</v>
+      </c>
+    </row>
+    <row r="861" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A861" t="s">
+        <v>2390</v>
+      </c>
+      <c r="B861" t="s">
+        <v>2391</v>
+      </c>
+      <c r="C861" t="s">
+        <v>2392</v>
+      </c>
+    </row>
+    <row r="862" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A862" t="s">
+        <v>2393</v>
+      </c>
+      <c r="B862" t="s">
+        <v>2394</v>
+      </c>
+      <c r="C862" t="s">
+        <v>2395</v>
+      </c>
+    </row>
+    <row r="863" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A863" t="s">
+        <v>2396</v>
+      </c>
+      <c r="B863" t="s">
+        <v>2397</v>
+      </c>
+      <c r="C863" t="s">
+        <v>2398</v>
+      </c>
+    </row>
+    <row r="864" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A864" t="s">
+        <v>2399</v>
+      </c>
+      <c r="B864" t="s">
+        <v>2400</v>
+      </c>
+      <c r="C864" t="s">
+        <v>2401</v>
+      </c>
+    </row>
+    <row r="865" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A865" t="s">
+        <v>2402</v>
+      </c>
+      <c r="B865" t="s">
+        <v>2403</v>
+      </c>
+      <c r="C865" t="s">
+        <v>2404</v>
+      </c>
+    </row>
+    <row r="866" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A866" t="s">
+        <v>2405</v>
+      </c>
+      <c r="B866" t="s">
+        <v>344</v>
+      </c>
+      <c r="C866" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="867" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A867" t="s">
+        <v>2406</v>
+      </c>
+      <c r="B867" t="s">
+        <v>2407</v>
+      </c>
+      <c r="C867" t="s">
+        <v>2408</v>
+      </c>
+    </row>
+    <row r="868" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A868" t="s">
+        <v>2409</v>
+      </c>
+      <c r="B868" t="s">
+        <v>2410</v>
+      </c>
+      <c r="C868" t="s">
+        <v>2411</v>
+      </c>
+    </row>
+    <row r="869" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A869" t="s">
+        <v>2412</v>
+      </c>
+      <c r="B869" t="s">
+        <v>2413</v>
+      </c>
+      <c r="C869" t="s">
+        <v>2414</v>
+      </c>
+    </row>
+    <row r="870" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A870" t="s">
+        <v>2415</v>
+      </c>
+      <c r="B870" t="s">
+        <v>2416</v>
+      </c>
+      <c r="C870" t="s">
+        <v>2417</v>
+      </c>
+    </row>
+    <row r="871" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A871" t="s">
+        <v>2418</v>
+      </c>
+      <c r="B871" t="s">
+        <v>2419</v>
+      </c>
+      <c r="C871" t="s">
+        <v>2420</v>
+      </c>
+    </row>
+    <row r="872" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A872" t="s">
+        <v>2421</v>
+      </c>
+      <c r="B872" t="s">
+        <v>2422</v>
+      </c>
+      <c r="C872" t="s">
+        <v>2423</v>
+      </c>
+    </row>
+    <row r="873" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A873" t="s">
+        <v>2424</v>
+      </c>
+      <c r="B873" t="s">
+        <v>2425</v>
+      </c>
+      <c r="C873" t="s">
+        <v>2426</v>
+      </c>
+    </row>
+    <row r="874" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A874" t="s">
+        <v>2427</v>
+      </c>
+      <c r="B874" t="s">
+        <v>2428</v>
+      </c>
+      <c r="C874" t="s">
+        <v>2429</v>
+      </c>
+    </row>
+    <row r="875" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A875" t="s">
+        <v>2430</v>
+      </c>
+      <c r="B875" t="s">
+        <v>2431</v>
+      </c>
+      <c r="C875" t="s">
+        <v>2432</v>
+      </c>
+    </row>
+    <row r="876" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A876" t="s">
+        <v>2433</v>
+      </c>
+      <c r="B876" t="s">
+        <v>2434</v>
+      </c>
+      <c r="C876" t="s">
+        <v>2435</v>
+      </c>
+    </row>
+    <row r="877" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A877" t="s">
+        <v>2436</v>
+      </c>
+      <c r="B877" t="s">
+        <v>2437</v>
+      </c>
+      <c r="C877" t="s">
+        <v>2438</v>
+      </c>
+    </row>
+    <row r="878" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A878" t="s">
+        <v>2439</v>
+      </c>
+      <c r="B878" t="s">
+        <v>359</v>
+      </c>
+      <c r="C878" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="879" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A879" t="s">
+        <v>2440</v>
+      </c>
+      <c r="B879" t="s">
+        <v>2441</v>
+      </c>
+      <c r="C879" t="s">
+        <v>2442</v>
+      </c>
+    </row>
+    <row r="880" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A880" t="s">
+        <v>2443</v>
+      </c>
+      <c r="B880" t="s">
+        <v>2444</v>
+      </c>
+      <c r="C880" t="s">
+        <v>2445</v>
+      </c>
+    </row>
+    <row r="881" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A881" t="s">
+        <v>2446</v>
+      </c>
+      <c r="B881" t="s">
+        <v>2447</v>
+      </c>
+      <c r="C881" t="s">
+        <v>2448</v>
+      </c>
+    </row>
+    <row r="882" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A882" t="s">
+        <v>2449</v>
+      </c>
+      <c r="B882" t="s">
+        <v>2450</v>
+      </c>
+      <c r="C882" t="s">
+        <v>2451</v>
+      </c>
+    </row>
+    <row r="883" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A883" t="s">
+        <v>2452</v>
+      </c>
+      <c r="B883" t="s">
+        <v>2453</v>
+      </c>
+      <c r="C883" t="s">
+        <v>2454</v>
+      </c>
+    </row>
+    <row r="884" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A884" t="s">
+        <v>2455</v>
+      </c>
+      <c r="B884" t="s">
+        <v>2284</v>
+      </c>
+      <c r="C884" t="s">
+        <v>2285</v>
+      </c>
+    </row>
+    <row r="885" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A885" t="s">
+        <v>2456</v>
+      </c>
+      <c r="B885" t="s">
+        <v>2457</v>
+      </c>
+      <c r="C885" t="s">
+        <v>2458</v>
+      </c>
+    </row>
+    <row r="886" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A886" t="s">
+        <v>2459</v>
+      </c>
+      <c r="B886" t="s">
+        <v>2460</v>
+      </c>
+      <c r="C886" t="s">
+        <v>2461</v>
+      </c>
+    </row>
+    <row r="887" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A887" t="s">
+        <v>2462</v>
+      </c>
+      <c r="B887" t="s">
+        <v>2463</v>
+      </c>
+      <c r="C887" t="s">
+        <v>2464</v>
+      </c>
+    </row>
+    <row r="888" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A888" t="s">
+        <v>2465</v>
+      </c>
+      <c r="B888" t="s">
+        <v>2466</v>
+      </c>
+      <c r="C888" t="s">
+        <v>2467</v>
+      </c>
+    </row>
+    <row r="889" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A889" t="s">
+        <v>2468</v>
+      </c>
+      <c r="B889" t="s">
+        <v>2469</v>
+      </c>
+      <c r="C889" t="s">
+        <v>2470</v>
+      </c>
+    </row>
+    <row r="890" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A890" t="s">
+        <v>2471</v>
+      </c>
+      <c r="B890" t="s">
+        <v>2472</v>
+      </c>
+      <c r="C890" t="s">
+        <v>2473</v>
+      </c>
+    </row>
+    <row r="891" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A891" t="s">
+        <v>2474</v>
+      </c>
+      <c r="B891" t="s">
+        <v>2472</v>
+      </c>
+      <c r="C891" t="s">
+        <v>2473</v>
+      </c>
+    </row>
+    <row r="892" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A892" t="s">
+        <v>2475</v>
+      </c>
+      <c r="B892" t="s">
+        <v>2476</v>
+      </c>
+      <c r="C892" t="s">
+        <v>2477</v>
+      </c>
+    </row>
+    <row r="893" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A893" t="s">
+        <v>2478</v>
+      </c>
+      <c r="B893" t="s">
+        <v>2479</v>
+      </c>
+      <c r="C893" t="s">
+        <v>2480</v>
+      </c>
+    </row>
+    <row r="894" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A894" t="s">
+        <v>2481</v>
+      </c>
+      <c r="B894" t="s">
+        <v>2482</v>
+      </c>
+      <c r="C894" t="s">
+        <v>2483</v>
+      </c>
+    </row>
+    <row r="895" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A895" t="s">
+        <v>2484</v>
+      </c>
+      <c r="B895" t="s">
+        <v>2485</v>
+      </c>
+      <c r="C895" t="s">
+        <v>2486</v>
+      </c>
+    </row>
+    <row r="896" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A896" t="s">
+        <v>2487</v>
+      </c>
+      <c r="B896" t="s">
+        <v>2488</v>
+      </c>
+      <c r="C896" t="s">
+        <v>2489</v>
+      </c>
+    </row>
+    <row r="897" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A897" t="s">
+        <v>2490</v>
+      </c>
+      <c r="B897" t="s">
+        <v>2491</v>
+      </c>
+      <c r="C897" t="s">
+        <v>2492</v>
+      </c>
+    </row>
+    <row r="898" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A898" t="s">
+        <v>2493</v>
+      </c>
+      <c r="B898" t="s">
+        <v>2494</v>
+      </c>
+      <c r="C898" t="s">
+        <v>2495</v>
+      </c>
+    </row>
+    <row r="899" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A899" t="s">
+        <v>2496</v>
+      </c>
+      <c r="B899" t="s">
+        <v>2497</v>
+      </c>
+      <c r="C899" t="s">
+        <v>2498</v>
+      </c>
+    </row>
+    <row r="900" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A900" t="s">
+        <v>2499</v>
+      </c>
+      <c r="B900" t="s">
+        <v>2500</v>
+      </c>
+      <c r="C900" t="s">
+        <v>2501</v>
+      </c>
+    </row>
+    <row r="901" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A901" t="s">
+        <v>2502</v>
+      </c>
+      <c r="B901" t="s">
+        <v>2503</v>
+      </c>
+      <c r="C901" t="s">
+        <v>2504</v>
+      </c>
+    </row>
+    <row r="902" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A902" t="s">
+        <v>2505</v>
+      </c>
+      <c r="B902" t="s">
+        <v>2506</v>
+      </c>
+      <c r="C902" t="s">
+        <v>2507</v>
+      </c>
+    </row>
+    <row r="903" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A903" t="s">
+        <v>2508</v>
+      </c>
+      <c r="B903" t="s">
+        <v>2167</v>
+      </c>
+      <c r="C903" t="s">
+        <v>2168</v>
+      </c>
+    </row>
+    <row r="904" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A904" t="s">
+        <v>2509</v>
+      </c>
+      <c r="B904" t="s">
+        <v>2167</v>
+      </c>
+      <c r="C904" t="s">
+        <v>2510</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>

</xml_diff>